<commit_message>
update to process more user friendly spreadsheet
created calc.R for conversion and calculation functions, moved some functions to utils.R or their own file.
</commit_message>
<xml_diff>
--- a/files/Templates/STICS_tabDataTemplate.xlsx
+++ b/files/Templates/STICS_tabDataTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Students\Maria\STICS\mkSTICSfiles\files\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marpo\Documents\Research\STICS\Code\mkSTICSfiles\files\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC7D4B4B-C5AD-4127-8C2C-C67F21656CB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D84D99-402B-4677-8B4F-001E1AAC34BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="usms" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="obs - usm1" sheetId="7" r:id="rId6"/>
     <sheet name="obs - usm2" sheetId="8" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="248">
   <si>
     <t>usm_name</t>
   </si>
@@ -756,19 +756,53 @@
   </si>
   <si>
     <t>mais.lai</t>
+  </si>
+  <si>
+    <t>HCCF_5</t>
+  </si>
+  <si>
+    <t>HMINF_5</t>
+  </si>
+  <si>
+    <t>DAF_5</t>
+  </si>
+  <si>
+    <t>typecailloux_5</t>
+  </si>
+  <si>
+    <t>cailloux_5</t>
+  </si>
+  <si>
+    <t>infil_5</t>
+  </si>
+  <si>
+    <t>epd_5</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>concrr</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -836,8 +870,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1048,6 +1087,12 @@
         <bgColor rgb="FFF7C9C9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor rgb="FFEDEDED"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="14">
     <border>
@@ -1172,19 +1217,6 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -1202,12 +1234,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1244,25 +1287,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1283,22 +1325,22 @@
     <xf numFmtId="0" fontId="0" fillId="17" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="24" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="22" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="22" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="24" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1307,95 +1349,126 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="26" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="23" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="23" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="25" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="23" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="29" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="29" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="31" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="32" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="33" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="28" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="31" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="34" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="34" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="31" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="35" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="35" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="30" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="33" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="36" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="28" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="36" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="31" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="34" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="34" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="31" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="35" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="35" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="30" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="36" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="27" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1806,72 +1879,72 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="43.90625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.81640625" customWidth="1"/>
-    <col min="3" max="3" width="22.81640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="22.81640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="14.08984375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.36328125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="43.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.77734375" customWidth="1"/>
+    <col min="3" max="3" width="22.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="22.77734375" style="9" customWidth="1"/>
+    <col min="5" max="5" width="14.109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.33203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="22.81640625" style="1" customWidth="1"/>
-    <col min="9" max="10" width="22.81640625" customWidth="1"/>
-    <col min="11" max="11" width="22.81640625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="22.81640625" customWidth="1"/>
-    <col min="13" max="13" width="60.08984375" customWidth="1"/>
-    <col min="14" max="14" width="22.81640625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="22.81640625" style="9" customWidth="1"/>
-    <col min="16" max="17" width="22.81640625" customWidth="1"/>
-    <col min="18" max="18" width="22.81640625" style="1" customWidth="1"/>
-    <col min="19" max="19" width="22.81640625" style="61" customWidth="1"/>
-    <col min="20" max="1025" width="10.54296875" customWidth="1"/>
+    <col min="8" max="8" width="22.77734375" style="1" customWidth="1"/>
+    <col min="9" max="10" width="22.77734375" customWidth="1"/>
+    <col min="11" max="11" width="22.77734375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="22.77734375" customWidth="1"/>
+    <col min="13" max="13" width="60.109375" customWidth="1"/>
+    <col min="14" max="14" width="22.77734375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="22.77734375" style="9" customWidth="1"/>
+    <col min="16" max="17" width="22.77734375" customWidth="1"/>
+    <col min="18" max="18" width="22.77734375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="22.77734375" style="59" customWidth="1"/>
+    <col min="20" max="1025" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="7" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="73" t="s">
+    <row r="1" spans="1:19" s="7" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="74" t="s">
+      <c r="B1" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="75" t="s">
+      <c r="C1" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="78" t="s">
+      <c r="D1" s="109" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="79" t="s">
+      <c r="E1" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="81" t="s">
+      <c r="F1" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="82" t="s">
+      <c r="G1" s="76" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="81" t="s">
+      <c r="H1" s="75" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="83" t="s">
+      <c r="I1" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="83" t="s">
+      <c r="J1" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="76" t="s">
+      <c r="K1" s="71" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="84" t="s">
+      <c r="L1" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="84" t="s">
+      <c r="M1" s="78" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="97" t="s">
+      <c r="O1" s="91" t="s">
         <v>14</v>
       </c>
       <c r="P1" s="5" t="s">
@@ -1883,19 +1956,36 @@
       <c r="R1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="80" t="s">
+      <c r="S1" s="74" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="E2" s="77"/>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="B2">
+        <v>105</v>
+      </c>
+      <c r="C2" s="1">
+        <v>325</v>
+      </c>
+      <c r="E2" s="72"/>
       <c r="N2" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="O2" s="96"/>
-      <c r="S2" s="60"/>
+      <c r="O2" s="90"/>
+      <c r="P2" t="s">
+        <v>246</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>246</v>
+      </c>
+      <c r="R2" t="s">
+        <v>246</v>
+      </c>
+      <c r="S2" t="s">
+        <v>246</v>
+      </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E3" s="9"/>
     </row>
   </sheetData>
@@ -1907,32 +1997,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AD2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" style="8" customWidth="1"/>
-    <col min="2" max="2" width="9.90625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" style="1" customWidth="1"/>
     <col min="3" max="3" width="13" style="9" customWidth="1"/>
-    <col min="4" max="4" width="10.1796875" customWidth="1"/>
-    <col min="5" max="5" width="15.1796875" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" customWidth="1"/>
-    <col min="7" max="7" width="33.90625" customWidth="1"/>
-    <col min="8" max="8" width="13.6328125" customWidth="1"/>
-    <col min="9" max="9" width="16.90625" customWidth="1"/>
-    <col min="10" max="10" width="18.54296875" style="1" customWidth="1"/>
-    <col min="11" max="14" width="18.6328125" customWidth="1"/>
-    <col min="15" max="15" width="18.6328125" style="1" customWidth="1"/>
-    <col min="16" max="19" width="7.08984375" customWidth="1"/>
-    <col min="20" max="20" width="7.08984375" style="1" customWidth="1"/>
-    <col min="21" max="24" width="9.90625" customWidth="1"/>
-    <col min="25" max="25" width="9.90625" style="1" customWidth="1"/>
-    <col min="26" max="29" width="9.6328125" customWidth="1"/>
-    <col min="30" max="30" width="9.6328125" style="8" customWidth="1"/>
-    <col min="31" max="1014" width="10.54296875" customWidth="1"/>
-    <col min="1015" max="1025" width="9.08984375" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" customWidth="1"/>
+    <col min="5" max="5" width="15.21875" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" customWidth="1"/>
+    <col min="7" max="7" width="33.88671875" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" customWidth="1"/>
+    <col min="9" max="9" width="16.88671875" customWidth="1"/>
+    <col min="10" max="10" width="18.5546875" style="1" customWidth="1"/>
+    <col min="11" max="14" width="18.6640625" customWidth="1"/>
+    <col min="15" max="15" width="18.6640625" style="1" customWidth="1"/>
+    <col min="16" max="19" width="7.109375" customWidth="1"/>
+    <col min="20" max="20" width="7.109375" style="1" customWidth="1"/>
+    <col min="21" max="24" width="9.88671875" customWidth="1"/>
+    <col min="25" max="25" width="9.88671875" style="1" customWidth="1"/>
+    <col min="26" max="29" width="9.6640625" customWidth="1"/>
+    <col min="30" max="30" width="9.6640625" style="8" customWidth="1"/>
+    <col min="31" max="1014" width="10.5546875" customWidth="1"/>
+    <col min="1015" max="1025" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="90" t="s">
+    <row r="1" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="84" t="s">
         <v>19</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -1977,53 +2067,53 @@
       <c r="O1" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="P1" s="91" t="s">
+      <c r="P1" s="85" t="s">
         <v>33</v>
       </c>
-      <c r="Q1" s="91" t="s">
+      <c r="Q1" s="85" t="s">
         <v>34</v>
       </c>
-      <c r="R1" s="91" t="s">
+      <c r="R1" s="85" t="s">
         <v>35</v>
       </c>
-      <c r="S1" s="91" t="s">
+      <c r="S1" s="85" t="s">
         <v>36</v>
       </c>
-      <c r="T1" s="92" t="s">
+      <c r="T1" s="86" t="s">
         <v>37</v>
       </c>
-      <c r="U1" s="93" t="s">
+      <c r="U1" s="87" t="s">
         <v>38</v>
       </c>
-      <c r="V1" s="93" t="s">
+      <c r="V1" s="87" t="s">
         <v>39</v>
       </c>
-      <c r="W1" s="93" t="s">
+      <c r="W1" s="87" t="s">
         <v>40</v>
       </c>
-      <c r="X1" s="93" t="s">
+      <c r="X1" s="87" t="s">
         <v>41</v>
       </c>
-      <c r="Y1" s="90" t="s">
+      <c r="Y1" s="84" t="s">
         <v>42</v>
       </c>
-      <c r="Z1" s="94" t="s">
+      <c r="Z1" s="88" t="s">
         <v>43</v>
       </c>
-      <c r="AA1" s="94" t="s">
+      <c r="AA1" s="88" t="s">
         <v>44</v>
       </c>
-      <c r="AB1" s="94" t="s">
+      <c r="AB1" s="88" t="s">
         <v>45</v>
       </c>
-      <c r="AC1" s="94" t="s">
+      <c r="AC1" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="AD1" s="95" t="s">
+      <c r="AD1" s="89" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="B2" s="1">
         <v>1</v>
       </c>
@@ -2066,16 +2156,26 @@
       <c r="O2" s="1">
         <v>0</v>
       </c>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="13"/>
-      <c r="S2" s="13"/>
-      <c r="T2" s="59"/>
+      <c r="P2" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="13">
+        <v>0</v>
+      </c>
+      <c r="R2" s="13">
+        <v>0</v>
+      </c>
+      <c r="S2" s="13">
+        <v>0</v>
+      </c>
+      <c r="T2" s="58">
+        <v>0</v>
+      </c>
       <c r="U2" s="13"/>
       <c r="V2" s="13"/>
       <c r="W2" s="13"/>
       <c r="X2" s="13"/>
-      <c r="Y2" s="59"/>
+      <c r="Y2" s="58"/>
       <c r="Z2" s="13"/>
       <c r="AA2" s="13"/>
       <c r="AB2" s="13"/>
@@ -2090,256 +2190,256 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:BO14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:BV14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.1796875" style="8" customWidth="1"/>
-    <col min="2" max="2" width="5.54296875" customWidth="1"/>
-    <col min="3" max="3" width="4.54296875" customWidth="1"/>
-    <col min="4" max="4" width="5.08984375" customWidth="1"/>
-    <col min="5" max="6" width="4.54296875" customWidth="1"/>
-    <col min="7" max="8" width="9.08984375" customWidth="1"/>
-    <col min="9" max="9" width="5.453125" style="15" customWidth="1"/>
-    <col min="10" max="13" width="8.36328125" style="15" customWidth="1"/>
-    <col min="14" max="14" width="14.6328125" style="15" customWidth="1"/>
-    <col min="15" max="33" width="8.36328125" style="15" customWidth="1"/>
-    <col min="34" max="34" width="8.36328125" style="58" customWidth="1"/>
-    <col min="35" max="38" width="8.36328125" style="15" customWidth="1"/>
-    <col min="39" max="39" width="14.6328125" style="15" customWidth="1"/>
-    <col min="40" max="41" width="8.36328125" style="15" customWidth="1"/>
-    <col min="42" max="42" width="8.36328125" style="58" customWidth="1"/>
-    <col min="43" max="49" width="8.36328125" style="15" customWidth="1"/>
-    <col min="50" max="50" width="8.36328125" style="58" customWidth="1"/>
-    <col min="51" max="57" width="8.36328125" style="15" customWidth="1"/>
-    <col min="58" max="58" width="8.36328125" style="58" customWidth="1"/>
-    <col min="59" max="63" width="8.36328125" style="15" customWidth="1"/>
-    <col min="64" max="65" width="10.54296875" style="15" customWidth="1"/>
-    <col min="66" max="66" width="10.54296875" style="58" customWidth="1"/>
-    <col min="67" max="67" width="8.36328125" style="67" customWidth="1"/>
-    <col min="68" max="73" width="10.54296875" customWidth="1"/>
-    <col min="74" max="74" width="12.54296875" customWidth="1"/>
-    <col min="75" max="254" width="10.54296875" customWidth="1"/>
-    <col min="255" max="255" width="9.453125" customWidth="1"/>
-    <col min="256" max="256" width="6.6328125" customWidth="1"/>
-    <col min="257" max="257" width="5.54296875" customWidth="1"/>
-    <col min="258" max="258" width="5.453125" customWidth="1"/>
-    <col min="259" max="259" width="5.6328125" customWidth="1"/>
-    <col min="260" max="260" width="4.6328125" customWidth="1"/>
-    <col min="261" max="261" width="6.90625" customWidth="1"/>
-    <col min="262" max="262" width="5.453125" customWidth="1"/>
-    <col min="263" max="263" width="4.6328125" customWidth="1"/>
+    <col min="1" max="1" width="10.21875" style="8" customWidth="1"/>
+    <col min="2" max="2" width="5.5546875" customWidth="1"/>
+    <col min="3" max="3" width="4.5546875" customWidth="1"/>
+    <col min="4" max="4" width="5.109375" customWidth="1"/>
+    <col min="5" max="6" width="4.5546875" customWidth="1"/>
+    <col min="7" max="8" width="9.109375" customWidth="1"/>
+    <col min="9" max="9" width="5.44140625" style="15" customWidth="1"/>
+    <col min="10" max="13" width="8.33203125" style="15" customWidth="1"/>
+    <col min="14" max="14" width="14.6640625" style="15" customWidth="1"/>
+    <col min="15" max="33" width="8.33203125" style="15" customWidth="1"/>
+    <col min="34" max="34" width="8.33203125" style="57" customWidth="1"/>
+    <col min="35" max="38" width="8.33203125" style="15" customWidth="1"/>
+    <col min="39" max="39" width="14.6640625" style="15" customWidth="1"/>
+    <col min="40" max="41" width="8.33203125" style="15" customWidth="1"/>
+    <col min="42" max="42" width="8.33203125" style="57" customWidth="1"/>
+    <col min="43" max="49" width="8.33203125" style="15" customWidth="1"/>
+    <col min="50" max="50" width="8.33203125" style="57" customWidth="1"/>
+    <col min="51" max="57" width="8.33203125" style="15" customWidth="1"/>
+    <col min="58" max="58" width="8.33203125" style="57" customWidth="1"/>
+    <col min="59" max="63" width="8.33203125" style="15" customWidth="1"/>
+    <col min="64" max="65" width="10.5546875" style="15" customWidth="1"/>
+    <col min="66" max="66" width="10.5546875" style="57" customWidth="1"/>
+    <col min="67" max="67" width="8.33203125" style="15" customWidth="1"/>
+    <col min="68" max="73" width="10.5546875" customWidth="1"/>
+    <col min="74" max="74" width="12.5546875" style="8" customWidth="1"/>
+    <col min="75" max="254" width="10.5546875" customWidth="1"/>
+    <col min="255" max="255" width="9.44140625" customWidth="1"/>
+    <col min="256" max="256" width="6.6640625" customWidth="1"/>
+    <col min="257" max="257" width="5.5546875" customWidth="1"/>
+    <col min="258" max="258" width="5.44140625" customWidth="1"/>
+    <col min="259" max="259" width="5.6640625" customWidth="1"/>
+    <col min="260" max="260" width="4.6640625" customWidth="1"/>
+    <col min="261" max="261" width="6.88671875" customWidth="1"/>
+    <col min="262" max="262" width="5.44140625" customWidth="1"/>
+    <col min="263" max="263" width="4.6640625" customWidth="1"/>
     <col min="264" max="264" width="5" customWidth="1"/>
-    <col min="265" max="265" width="6.1796875" customWidth="1"/>
-    <col min="266" max="266" width="6.453125" customWidth="1"/>
-    <col min="267" max="267" width="7.08984375" customWidth="1"/>
-    <col min="268" max="268" width="5.54296875" customWidth="1"/>
-    <col min="269" max="269" width="5.6328125" customWidth="1"/>
-    <col min="270" max="270" width="6.54296875" customWidth="1"/>
-    <col min="271" max="271" width="6.453125" customWidth="1"/>
+    <col min="265" max="265" width="6.21875" customWidth="1"/>
+    <col min="266" max="266" width="6.44140625" customWidth="1"/>
+    <col min="267" max="267" width="7.109375" customWidth="1"/>
+    <col min="268" max="268" width="5.5546875" customWidth="1"/>
+    <col min="269" max="269" width="5.6640625" customWidth="1"/>
+    <col min="270" max="270" width="6.5546875" customWidth="1"/>
+    <col min="271" max="271" width="6.44140625" customWidth="1"/>
     <col min="272" max="272" width="6" customWidth="1"/>
-    <col min="273" max="273" width="5.08984375" customWidth="1"/>
-    <col min="274" max="274" width="6.54296875" customWidth="1"/>
-    <col min="275" max="277" width="5.90625" customWidth="1"/>
-    <col min="278" max="278" width="5.6328125" customWidth="1"/>
-    <col min="279" max="279" width="6.08984375" customWidth="1"/>
-    <col min="280" max="280" width="8.1796875" customWidth="1"/>
-    <col min="281" max="281" width="6.90625" customWidth="1"/>
-    <col min="282" max="282" width="6.6328125" customWidth="1"/>
-    <col min="283" max="283" width="5.08984375" customWidth="1"/>
-    <col min="284" max="284" width="6.54296875" customWidth="1"/>
-    <col min="285" max="285" width="8.08984375" customWidth="1"/>
-    <col min="286" max="287" width="5.90625" customWidth="1"/>
-    <col min="288" max="288" width="5.6328125" customWidth="1"/>
+    <col min="273" max="273" width="5.109375" customWidth="1"/>
+    <col min="274" max="274" width="6.5546875" customWidth="1"/>
+    <col min="275" max="277" width="5.88671875" customWidth="1"/>
+    <col min="278" max="278" width="5.6640625" customWidth="1"/>
+    <col min="279" max="279" width="6.109375" customWidth="1"/>
+    <col min="280" max="280" width="8.21875" customWidth="1"/>
+    <col min="281" max="281" width="6.88671875" customWidth="1"/>
+    <col min="282" max="282" width="6.6640625" customWidth="1"/>
+    <col min="283" max="283" width="5.109375" customWidth="1"/>
+    <col min="284" max="284" width="6.5546875" customWidth="1"/>
+    <col min="285" max="285" width="8.109375" customWidth="1"/>
+    <col min="286" max="287" width="5.88671875" customWidth="1"/>
+    <col min="288" max="288" width="5.6640625" customWidth="1"/>
     <col min="289" max="289" width="6" customWidth="1"/>
-    <col min="290" max="290" width="7.1796875" customWidth="1"/>
-    <col min="291" max="291" width="6.90625" customWidth="1"/>
-    <col min="292" max="292" width="6.6328125" customWidth="1"/>
-    <col min="293" max="293" width="5.08984375" customWidth="1"/>
-    <col min="294" max="294" width="6.54296875" customWidth="1"/>
-    <col min="295" max="295" width="8.08984375" customWidth="1"/>
-    <col min="296" max="297" width="5.90625" customWidth="1"/>
-    <col min="298" max="298" width="5.6328125" customWidth="1"/>
-    <col min="299" max="299" width="6.453125" customWidth="1"/>
-    <col min="300" max="300" width="9.1796875" customWidth="1"/>
-    <col min="301" max="301" width="6.90625" customWidth="1"/>
-    <col min="302" max="302" width="6.6328125" customWidth="1"/>
-    <col min="303" max="303" width="5.08984375" customWidth="1"/>
-    <col min="304" max="304" width="6.54296875" customWidth="1"/>
-    <col min="305" max="305" width="8.08984375" customWidth="1"/>
-    <col min="306" max="307" width="5.90625" customWidth="1"/>
-    <col min="308" max="308" width="5.6328125" customWidth="1"/>
-    <col min="309" max="309" width="7.1796875" customWidth="1"/>
-    <col min="310" max="310" width="9.6328125" customWidth="1"/>
-    <col min="311" max="311" width="6.90625" customWidth="1"/>
-    <col min="312" max="312" width="6.6328125" customWidth="1"/>
-    <col min="313" max="313" width="5.08984375" customWidth="1"/>
-    <col min="314" max="314" width="6.54296875" customWidth="1"/>
-    <col min="315" max="315" width="8.08984375" customWidth="1"/>
-    <col min="316" max="317" width="5.90625" customWidth="1"/>
-    <col min="318" max="318" width="5.6328125" customWidth="1"/>
+    <col min="290" max="290" width="7.21875" customWidth="1"/>
+    <col min="291" max="291" width="6.88671875" customWidth="1"/>
+    <col min="292" max="292" width="6.6640625" customWidth="1"/>
+    <col min="293" max="293" width="5.109375" customWidth="1"/>
+    <col min="294" max="294" width="6.5546875" customWidth="1"/>
+    <col min="295" max="295" width="8.109375" customWidth="1"/>
+    <col min="296" max="297" width="5.88671875" customWidth="1"/>
+    <col min="298" max="298" width="5.6640625" customWidth="1"/>
+    <col min="299" max="299" width="6.44140625" customWidth="1"/>
+    <col min="300" max="300" width="9.21875" customWidth="1"/>
+    <col min="301" max="301" width="6.88671875" customWidth="1"/>
+    <col min="302" max="302" width="6.6640625" customWidth="1"/>
+    <col min="303" max="303" width="5.109375" customWidth="1"/>
+    <col min="304" max="304" width="6.5546875" customWidth="1"/>
+    <col min="305" max="305" width="8.109375" customWidth="1"/>
+    <col min="306" max="307" width="5.88671875" customWidth="1"/>
+    <col min="308" max="308" width="5.6640625" customWidth="1"/>
+    <col min="309" max="309" width="7.21875" customWidth="1"/>
+    <col min="310" max="310" width="9.6640625" customWidth="1"/>
+    <col min="311" max="311" width="6.88671875" customWidth="1"/>
+    <col min="312" max="312" width="6.6640625" customWidth="1"/>
+    <col min="313" max="313" width="5.109375" customWidth="1"/>
+    <col min="314" max="314" width="6.5546875" customWidth="1"/>
+    <col min="315" max="315" width="8.109375" customWidth="1"/>
+    <col min="316" max="317" width="5.88671875" customWidth="1"/>
+    <col min="318" max="318" width="5.6640625" customWidth="1"/>
     <col min="319" max="320" width="9" customWidth="1"/>
-    <col min="321" max="321" width="6.90625" customWidth="1"/>
-    <col min="322" max="322" width="6.6328125" customWidth="1"/>
-    <col min="323" max="329" width="10.54296875" customWidth="1"/>
-    <col min="330" max="330" width="12.54296875" customWidth="1"/>
-    <col min="331" max="510" width="10.54296875" customWidth="1"/>
-    <col min="511" max="511" width="9.453125" customWidth="1"/>
-    <col min="512" max="512" width="6.6328125" customWidth="1"/>
-    <col min="513" max="513" width="5.54296875" customWidth="1"/>
-    <col min="514" max="514" width="5.453125" customWidth="1"/>
-    <col min="515" max="515" width="5.6328125" customWidth="1"/>
-    <col min="516" max="516" width="4.6328125" customWidth="1"/>
-    <col min="517" max="517" width="6.90625" customWidth="1"/>
-    <col min="518" max="518" width="5.453125" customWidth="1"/>
-    <col min="519" max="519" width="4.6328125" customWidth="1"/>
+    <col min="321" max="321" width="6.88671875" customWidth="1"/>
+    <col min="322" max="322" width="6.6640625" customWidth="1"/>
+    <col min="323" max="329" width="10.5546875" customWidth="1"/>
+    <col min="330" max="330" width="12.5546875" customWidth="1"/>
+    <col min="331" max="510" width="10.5546875" customWidth="1"/>
+    <col min="511" max="511" width="9.44140625" customWidth="1"/>
+    <col min="512" max="512" width="6.6640625" customWidth="1"/>
+    <col min="513" max="513" width="5.5546875" customWidth="1"/>
+    <col min="514" max="514" width="5.44140625" customWidth="1"/>
+    <col min="515" max="515" width="5.6640625" customWidth="1"/>
+    <col min="516" max="516" width="4.6640625" customWidth="1"/>
+    <col min="517" max="517" width="6.88671875" customWidth="1"/>
+    <col min="518" max="518" width="5.44140625" customWidth="1"/>
+    <col min="519" max="519" width="4.6640625" customWidth="1"/>
     <col min="520" max="520" width="5" customWidth="1"/>
-    <col min="521" max="521" width="6.1796875" customWidth="1"/>
-    <col min="522" max="522" width="6.453125" customWidth="1"/>
-    <col min="523" max="523" width="7.08984375" customWidth="1"/>
-    <col min="524" max="524" width="5.54296875" customWidth="1"/>
-    <col min="525" max="525" width="5.6328125" customWidth="1"/>
-    <col min="526" max="526" width="6.54296875" customWidth="1"/>
-    <col min="527" max="527" width="6.453125" customWidth="1"/>
+    <col min="521" max="521" width="6.21875" customWidth="1"/>
+    <col min="522" max="522" width="6.44140625" customWidth="1"/>
+    <col min="523" max="523" width="7.109375" customWidth="1"/>
+    <col min="524" max="524" width="5.5546875" customWidth="1"/>
+    <col min="525" max="525" width="5.6640625" customWidth="1"/>
+    <col min="526" max="526" width="6.5546875" customWidth="1"/>
+    <col min="527" max="527" width="6.44140625" customWidth="1"/>
     <col min="528" max="528" width="6" customWidth="1"/>
-    <col min="529" max="529" width="5.08984375" customWidth="1"/>
-    <col min="530" max="530" width="6.54296875" customWidth="1"/>
-    <col min="531" max="533" width="5.90625" customWidth="1"/>
-    <col min="534" max="534" width="5.6328125" customWidth="1"/>
-    <col min="535" max="535" width="6.08984375" customWidth="1"/>
-    <col min="536" max="536" width="8.1796875" customWidth="1"/>
-    <col min="537" max="537" width="6.90625" customWidth="1"/>
-    <col min="538" max="538" width="6.6328125" customWidth="1"/>
-    <col min="539" max="539" width="5.08984375" customWidth="1"/>
-    <col min="540" max="540" width="6.54296875" customWidth="1"/>
-    <col min="541" max="541" width="8.08984375" customWidth="1"/>
-    <col min="542" max="543" width="5.90625" customWidth="1"/>
-    <col min="544" max="544" width="5.6328125" customWidth="1"/>
+    <col min="529" max="529" width="5.109375" customWidth="1"/>
+    <col min="530" max="530" width="6.5546875" customWidth="1"/>
+    <col min="531" max="533" width="5.88671875" customWidth="1"/>
+    <col min="534" max="534" width="5.6640625" customWidth="1"/>
+    <col min="535" max="535" width="6.109375" customWidth="1"/>
+    <col min="536" max="536" width="8.21875" customWidth="1"/>
+    <col min="537" max="537" width="6.88671875" customWidth="1"/>
+    <col min="538" max="538" width="6.6640625" customWidth="1"/>
+    <col min="539" max="539" width="5.109375" customWidth="1"/>
+    <col min="540" max="540" width="6.5546875" customWidth="1"/>
+    <col min="541" max="541" width="8.109375" customWidth="1"/>
+    <col min="542" max="543" width="5.88671875" customWidth="1"/>
+    <col min="544" max="544" width="5.6640625" customWidth="1"/>
     <col min="545" max="545" width="6" customWidth="1"/>
-    <col min="546" max="546" width="7.1796875" customWidth="1"/>
-    <col min="547" max="547" width="6.90625" customWidth="1"/>
-    <col min="548" max="548" width="6.6328125" customWidth="1"/>
-    <col min="549" max="549" width="5.08984375" customWidth="1"/>
-    <col min="550" max="550" width="6.54296875" customWidth="1"/>
-    <col min="551" max="551" width="8.08984375" customWidth="1"/>
-    <col min="552" max="553" width="5.90625" customWidth="1"/>
-    <col min="554" max="554" width="5.6328125" customWidth="1"/>
-    <col min="555" max="555" width="6.453125" customWidth="1"/>
-    <col min="556" max="556" width="9.1796875" customWidth="1"/>
-    <col min="557" max="557" width="6.90625" customWidth="1"/>
-    <col min="558" max="558" width="6.6328125" customWidth="1"/>
-    <col min="559" max="559" width="5.08984375" customWidth="1"/>
-    <col min="560" max="560" width="6.54296875" customWidth="1"/>
-    <col min="561" max="561" width="8.08984375" customWidth="1"/>
-    <col min="562" max="563" width="5.90625" customWidth="1"/>
-    <col min="564" max="564" width="5.6328125" customWidth="1"/>
-    <col min="565" max="565" width="7.1796875" customWidth="1"/>
-    <col min="566" max="566" width="9.6328125" customWidth="1"/>
-    <col min="567" max="567" width="6.90625" customWidth="1"/>
-    <col min="568" max="568" width="6.6328125" customWidth="1"/>
-    <col min="569" max="569" width="5.08984375" customWidth="1"/>
-    <col min="570" max="570" width="6.54296875" customWidth="1"/>
-    <col min="571" max="571" width="8.08984375" customWidth="1"/>
-    <col min="572" max="573" width="5.90625" customWidth="1"/>
-    <col min="574" max="574" width="5.6328125" customWidth="1"/>
+    <col min="546" max="546" width="7.21875" customWidth="1"/>
+    <col min="547" max="547" width="6.88671875" customWidth="1"/>
+    <col min="548" max="548" width="6.6640625" customWidth="1"/>
+    <col min="549" max="549" width="5.109375" customWidth="1"/>
+    <col min="550" max="550" width="6.5546875" customWidth="1"/>
+    <col min="551" max="551" width="8.109375" customWidth="1"/>
+    <col min="552" max="553" width="5.88671875" customWidth="1"/>
+    <col min="554" max="554" width="5.6640625" customWidth="1"/>
+    <col min="555" max="555" width="6.44140625" customWidth="1"/>
+    <col min="556" max="556" width="9.21875" customWidth="1"/>
+    <col min="557" max="557" width="6.88671875" customWidth="1"/>
+    <col min="558" max="558" width="6.6640625" customWidth="1"/>
+    <col min="559" max="559" width="5.109375" customWidth="1"/>
+    <col min="560" max="560" width="6.5546875" customWidth="1"/>
+    <col min="561" max="561" width="8.109375" customWidth="1"/>
+    <col min="562" max="563" width="5.88671875" customWidth="1"/>
+    <col min="564" max="564" width="5.6640625" customWidth="1"/>
+    <col min="565" max="565" width="7.21875" customWidth="1"/>
+    <col min="566" max="566" width="9.6640625" customWidth="1"/>
+    <col min="567" max="567" width="6.88671875" customWidth="1"/>
+    <col min="568" max="568" width="6.6640625" customWidth="1"/>
+    <col min="569" max="569" width="5.109375" customWidth="1"/>
+    <col min="570" max="570" width="6.5546875" customWidth="1"/>
+    <col min="571" max="571" width="8.109375" customWidth="1"/>
+    <col min="572" max="573" width="5.88671875" customWidth="1"/>
+    <col min="574" max="574" width="5.6640625" customWidth="1"/>
     <col min="575" max="576" width="9" customWidth="1"/>
-    <col min="577" max="577" width="6.90625" customWidth="1"/>
-    <col min="578" max="578" width="6.6328125" customWidth="1"/>
-    <col min="579" max="585" width="10.54296875" customWidth="1"/>
-    <col min="586" max="586" width="12.54296875" customWidth="1"/>
-    <col min="587" max="766" width="10.54296875" customWidth="1"/>
-    <col min="767" max="767" width="9.453125" customWidth="1"/>
-    <col min="768" max="768" width="6.6328125" customWidth="1"/>
-    <col min="769" max="769" width="5.54296875" customWidth="1"/>
-    <col min="770" max="770" width="5.453125" customWidth="1"/>
-    <col min="771" max="771" width="5.6328125" customWidth="1"/>
-    <col min="772" max="772" width="4.6328125" customWidth="1"/>
-    <col min="773" max="773" width="6.90625" customWidth="1"/>
-    <col min="774" max="774" width="5.453125" customWidth="1"/>
-    <col min="775" max="775" width="4.6328125" customWidth="1"/>
+    <col min="577" max="577" width="6.88671875" customWidth="1"/>
+    <col min="578" max="578" width="6.6640625" customWidth="1"/>
+    <col min="579" max="585" width="10.5546875" customWidth="1"/>
+    <col min="586" max="586" width="12.5546875" customWidth="1"/>
+    <col min="587" max="766" width="10.5546875" customWidth="1"/>
+    <col min="767" max="767" width="9.44140625" customWidth="1"/>
+    <col min="768" max="768" width="6.6640625" customWidth="1"/>
+    <col min="769" max="769" width="5.5546875" customWidth="1"/>
+    <col min="770" max="770" width="5.44140625" customWidth="1"/>
+    <col min="771" max="771" width="5.6640625" customWidth="1"/>
+    <col min="772" max="772" width="4.6640625" customWidth="1"/>
+    <col min="773" max="773" width="6.88671875" customWidth="1"/>
+    <col min="774" max="774" width="5.44140625" customWidth="1"/>
+    <col min="775" max="775" width="4.6640625" customWidth="1"/>
     <col min="776" max="776" width="5" customWidth="1"/>
-    <col min="777" max="777" width="6.1796875" customWidth="1"/>
-    <col min="778" max="778" width="6.453125" customWidth="1"/>
-    <col min="779" max="779" width="7.08984375" customWidth="1"/>
-    <col min="780" max="780" width="5.54296875" customWidth="1"/>
-    <col min="781" max="781" width="5.6328125" customWidth="1"/>
-    <col min="782" max="782" width="6.54296875" customWidth="1"/>
-    <col min="783" max="783" width="6.453125" customWidth="1"/>
+    <col min="777" max="777" width="6.21875" customWidth="1"/>
+    <col min="778" max="778" width="6.44140625" customWidth="1"/>
+    <col min="779" max="779" width="7.109375" customWidth="1"/>
+    <col min="780" max="780" width="5.5546875" customWidth="1"/>
+    <col min="781" max="781" width="5.6640625" customWidth="1"/>
+    <col min="782" max="782" width="6.5546875" customWidth="1"/>
+    <col min="783" max="783" width="6.44140625" customWidth="1"/>
     <col min="784" max="784" width="6" customWidth="1"/>
-    <col min="785" max="785" width="5.08984375" customWidth="1"/>
-    <col min="786" max="786" width="6.54296875" customWidth="1"/>
-    <col min="787" max="789" width="5.90625" customWidth="1"/>
-    <col min="790" max="790" width="5.6328125" customWidth="1"/>
-    <col min="791" max="791" width="6.08984375" customWidth="1"/>
-    <col min="792" max="792" width="8.1796875" customWidth="1"/>
-    <col min="793" max="793" width="6.90625" customWidth="1"/>
-    <col min="794" max="794" width="6.6328125" customWidth="1"/>
-    <col min="795" max="795" width="5.08984375" customWidth="1"/>
-    <col min="796" max="796" width="6.54296875" customWidth="1"/>
-    <col min="797" max="797" width="8.08984375" customWidth="1"/>
-    <col min="798" max="799" width="5.90625" customWidth="1"/>
-    <col min="800" max="800" width="5.6328125" customWidth="1"/>
+    <col min="785" max="785" width="5.109375" customWidth="1"/>
+    <col min="786" max="786" width="6.5546875" customWidth="1"/>
+    <col min="787" max="789" width="5.88671875" customWidth="1"/>
+    <col min="790" max="790" width="5.6640625" customWidth="1"/>
+    <col min="791" max="791" width="6.109375" customWidth="1"/>
+    <col min="792" max="792" width="8.21875" customWidth="1"/>
+    <col min="793" max="793" width="6.88671875" customWidth="1"/>
+    <col min="794" max="794" width="6.6640625" customWidth="1"/>
+    <col min="795" max="795" width="5.109375" customWidth="1"/>
+    <col min="796" max="796" width="6.5546875" customWidth="1"/>
+    <col min="797" max="797" width="8.109375" customWidth="1"/>
+    <col min="798" max="799" width="5.88671875" customWidth="1"/>
+    <col min="800" max="800" width="5.6640625" customWidth="1"/>
     <col min="801" max="801" width="6" customWidth="1"/>
-    <col min="802" max="802" width="7.1796875" customWidth="1"/>
-    <col min="803" max="803" width="6.90625" customWidth="1"/>
-    <col min="804" max="804" width="6.6328125" customWidth="1"/>
-    <col min="805" max="805" width="5.08984375" customWidth="1"/>
-    <col min="806" max="806" width="6.54296875" customWidth="1"/>
-    <col min="807" max="807" width="8.08984375" customWidth="1"/>
-    <col min="808" max="809" width="5.90625" customWidth="1"/>
-    <col min="810" max="810" width="5.6328125" customWidth="1"/>
-    <col min="811" max="811" width="6.453125" customWidth="1"/>
-    <col min="812" max="812" width="9.1796875" customWidth="1"/>
-    <col min="813" max="813" width="6.90625" customWidth="1"/>
-    <col min="814" max="814" width="6.6328125" customWidth="1"/>
-    <col min="815" max="815" width="5.08984375" customWidth="1"/>
-    <col min="816" max="816" width="6.54296875" customWidth="1"/>
-    <col min="817" max="817" width="8.08984375" customWidth="1"/>
-    <col min="818" max="819" width="5.90625" customWidth="1"/>
-    <col min="820" max="820" width="5.6328125" customWidth="1"/>
-    <col min="821" max="821" width="7.1796875" customWidth="1"/>
-    <col min="822" max="822" width="9.6328125" customWidth="1"/>
-    <col min="823" max="823" width="6.90625" customWidth="1"/>
-    <col min="824" max="824" width="6.6328125" customWidth="1"/>
-    <col min="825" max="825" width="5.08984375" customWidth="1"/>
-    <col min="826" max="826" width="6.54296875" customWidth="1"/>
-    <col min="827" max="827" width="8.08984375" customWidth="1"/>
-    <col min="828" max="829" width="5.90625" customWidth="1"/>
-    <col min="830" max="830" width="5.6328125" customWidth="1"/>
+    <col min="802" max="802" width="7.21875" customWidth="1"/>
+    <col min="803" max="803" width="6.88671875" customWidth="1"/>
+    <col min="804" max="804" width="6.6640625" customWidth="1"/>
+    <col min="805" max="805" width="5.109375" customWidth="1"/>
+    <col min="806" max="806" width="6.5546875" customWidth="1"/>
+    <col min="807" max="807" width="8.109375" customWidth="1"/>
+    <col min="808" max="809" width="5.88671875" customWidth="1"/>
+    <col min="810" max="810" width="5.6640625" customWidth="1"/>
+    <col min="811" max="811" width="6.44140625" customWidth="1"/>
+    <col min="812" max="812" width="9.21875" customWidth="1"/>
+    <col min="813" max="813" width="6.88671875" customWidth="1"/>
+    <col min="814" max="814" width="6.6640625" customWidth="1"/>
+    <col min="815" max="815" width="5.109375" customWidth="1"/>
+    <col min="816" max="816" width="6.5546875" customWidth="1"/>
+    <col min="817" max="817" width="8.109375" customWidth="1"/>
+    <col min="818" max="819" width="5.88671875" customWidth="1"/>
+    <col min="820" max="820" width="5.6640625" customWidth="1"/>
+    <col min="821" max="821" width="7.21875" customWidth="1"/>
+    <col min="822" max="822" width="9.6640625" customWidth="1"/>
+    <col min="823" max="823" width="6.88671875" customWidth="1"/>
+    <col min="824" max="824" width="6.6640625" customWidth="1"/>
+    <col min="825" max="825" width="5.109375" customWidth="1"/>
+    <col min="826" max="826" width="6.5546875" customWidth="1"/>
+    <col min="827" max="827" width="8.109375" customWidth="1"/>
+    <col min="828" max="829" width="5.88671875" customWidth="1"/>
+    <col min="830" max="830" width="5.6640625" customWidth="1"/>
     <col min="831" max="832" width="9" customWidth="1"/>
-    <col min="833" max="833" width="6.90625" customWidth="1"/>
-    <col min="834" max="834" width="6.6328125" customWidth="1"/>
-    <col min="835" max="841" width="10.54296875" customWidth="1"/>
-    <col min="842" max="842" width="12.54296875" customWidth="1"/>
-    <col min="843" max="1018" width="10.54296875" customWidth="1"/>
-    <col min="1019" max="1025" width="9.08984375" customWidth="1"/>
+    <col min="833" max="833" width="6.88671875" customWidth="1"/>
+    <col min="834" max="834" width="6.6640625" customWidth="1"/>
+    <col min="835" max="841" width="10.5546875" customWidth="1"/>
+    <col min="842" max="842" width="12.5546875" customWidth="1"/>
+    <col min="843" max="1018" width="10.5546875" customWidth="1"/>
+    <col min="1019" max="1025" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:67" s="19" customFormat="1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="85" t="s">
+    <row r="1" spans="1:74" s="19" customFormat="1" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="79" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="86" t="s">
+      <c r="B1" s="80" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="86" t="s">
+      <c r="C1" s="80" t="s">
         <v>51</v>
       </c>
-      <c r="D1" s="86" t="s">
+      <c r="D1" s="80" t="s">
         <v>52</v>
       </c>
       <c r="E1" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="F1" s="87" t="s">
+      <c r="F1" s="81" t="s">
         <v>54</v>
       </c>
-      <c r="G1" s="87" t="s">
+      <c r="G1" s="92" t="s">
         <v>55</v>
       </c>
-      <c r="H1" s="87" t="s">
+      <c r="H1" s="81" t="s">
         <v>56</v>
       </c>
-      <c r="I1" s="87" t="s">
+      <c r="I1" s="81" t="s">
         <v>57</v>
       </c>
       <c r="J1" s="16" t="s">
@@ -2363,7 +2463,7 @@
       <c r="P1" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="Q1" s="87" t="s">
+      <c r="Q1" s="81" t="s">
         <v>65</v>
       </c>
       <c r="R1" s="16" t="s">
@@ -2414,19 +2514,19 @@
       <c r="AG1" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="AH1" s="63" t="s">
+      <c r="AH1" s="60" t="s">
         <v>82</v>
       </c>
-      <c r="AI1" s="88" t="s">
+      <c r="AI1" s="82" t="s">
         <v>83</v>
       </c>
-      <c r="AJ1" s="88" t="s">
+      <c r="AJ1" s="82" t="s">
         <v>84</v>
       </c>
-      <c r="AK1" s="88" t="s">
+      <c r="AK1" s="82" t="s">
         <v>85</v>
       </c>
-      <c r="AL1" s="88" t="s">
+      <c r="AL1" s="82" t="s">
         <v>86</v>
       </c>
       <c r="AM1" s="17" t="s">
@@ -2438,19 +2538,19 @@
       <c r="AO1" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="AP1" s="64" t="s">
+      <c r="AP1" s="61" t="s">
         <v>90</v>
       </c>
-      <c r="AQ1" s="89" t="s">
+      <c r="AQ1" s="83" t="s">
         <v>91</v>
       </c>
-      <c r="AR1" s="89" t="s">
+      <c r="AR1" s="83" t="s">
         <v>92</v>
       </c>
-      <c r="AS1" s="89" t="s">
+      <c r="AS1" s="83" t="s">
         <v>93</v>
       </c>
-      <c r="AT1" s="89" t="s">
+      <c r="AT1" s="83" t="s">
         <v>94</v>
       </c>
       <c r="AU1" s="18" t="s">
@@ -2462,19 +2562,19 @@
       <c r="AW1" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="AX1" s="65" t="s">
+      <c r="AX1" s="62" t="s">
         <v>98</v>
       </c>
-      <c r="AY1" s="88" t="s">
+      <c r="AY1" s="82" t="s">
         <v>99</v>
       </c>
-      <c r="AZ1" s="88" t="s">
+      <c r="AZ1" s="82" t="s">
         <v>100</v>
       </c>
-      <c r="BA1" s="88" t="s">
+      <c r="BA1" s="82" t="s">
         <v>101</v>
       </c>
-      <c r="BB1" s="88" t="s">
+      <c r="BB1" s="82" t="s">
         <v>102</v>
       </c>
       <c r="BC1" s="17" t="s">
@@ -2486,19 +2586,19 @@
       <c r="BE1" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="BF1" s="64" t="s">
+      <c r="BF1" s="61" t="s">
         <v>106</v>
       </c>
-      <c r="BG1" s="89" t="s">
+      <c r="BG1" s="83" t="s">
         <v>107</v>
       </c>
-      <c r="BH1" s="89" t="s">
+      <c r="BH1" s="83" t="s">
         <v>108</v>
       </c>
-      <c r="BI1" s="89" t="s">
+      <c r="BI1" s="83" t="s">
         <v>109</v>
       </c>
-      <c r="BJ1" s="89" t="s">
+      <c r="BJ1" s="83" t="s">
         <v>110</v>
       </c>
       <c r="BK1" s="18" t="s">
@@ -2510,25 +2610,44 @@
       <c r="BM1" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="BN1" s="65" t="s">
+      <c r="BN1" s="93" t="s">
         <v>114</v>
       </c>
-      <c r="BO1" s="65" t="s">
+      <c r="BO1" s="94" t="s">
         <v>115</v>
       </c>
+      <c r="BP1" s="96" t="s">
+        <v>239</v>
+      </c>
+      <c r="BQ1" s="96" t="s">
+        <v>240</v>
+      </c>
+      <c r="BR1" s="96" t="s">
+        <v>241</v>
+      </c>
+      <c r="BS1" s="94" t="s">
+        <v>242</v>
+      </c>
+      <c r="BT1" s="94" t="s">
+        <v>243</v>
+      </c>
+      <c r="BU1" s="94" t="s">
+        <v>244</v>
+      </c>
+      <c r="BV1" s="95" t="s">
+        <v>245</v>
+      </c>
     </row>
-    <row r="2" spans="1:67" s="13" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="62"/>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2"/>
+    <row r="2" spans="1:74" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="97"/>
+      <c r="D2" s="15"/>
       <c r="E2" s="20">
-        <v>1</v>
-      </c>
-      <c r="F2" s="20"/>
-      <c r="G2"/>
+        <v>0</v>
+      </c>
+      <c r="G2" s="15">
+        <v>0.01</v>
+      </c>
       <c r="H2" s="21"/>
-      <c r="I2" s="20"/>
       <c r="J2" s="20">
         <v>0</v>
       </c>
@@ -2550,7 +2669,6 @@
       <c r="P2" s="20">
         <v>0.01</v>
       </c>
-      <c r="Q2" s="20"/>
       <c r="R2" s="20">
         <v>0.65</v>
       </c>
@@ -2599,87 +2717,156 @@
       <c r="AG2" s="20">
         <v>20</v>
       </c>
-      <c r="AH2" s="57">
+      <c r="AH2" s="56">
         <v>2</v>
       </c>
-      <c r="AI2" s="22"/>
-      <c r="AJ2"/>
-      <c r="AK2"/>
-      <c r="AL2"/>
-      <c r="AM2">
+      <c r="AI2" s="98"/>
+      <c r="AM2" s="15">
         <v>1</v>
       </c>
-      <c r="AN2">
+      <c r="AN2" s="15">
         <v>0</v>
       </c>
-      <c r="AO2">
+      <c r="AO2" s="15">
         <v>50</v>
       </c>
-      <c r="AP2" s="1">
+      <c r="AP2" s="57">
         <v>10</v>
       </c>
-      <c r="AQ2" s="22"/>
-      <c r="AR2"/>
-      <c r="AS2"/>
-      <c r="AU2" s="13">
+      <c r="AQ2" s="98"/>
+      <c r="AR2" s="15"/>
+      <c r="AS2" s="15"/>
+      <c r="AU2" s="20">
         <v>1</v>
       </c>
-      <c r="AV2" s="13">
+      <c r="AV2" s="20">
         <v>0</v>
       </c>
-      <c r="AW2" s="13">
+      <c r="AW2" s="20">
         <v>50</v>
       </c>
-      <c r="AX2" s="59">
+      <c r="AX2" s="56">
         <v>10</v>
       </c>
-      <c r="AY2" s="22"/>
-      <c r="AZ2"/>
-      <c r="BA2"/>
-      <c r="BC2">
+      <c r="AY2" s="98"/>
+      <c r="BC2" s="15">
         <v>1</v>
       </c>
-      <c r="BD2">
+      <c r="BD2" s="15">
         <v>0</v>
       </c>
-      <c r="BE2">
+      <c r="BE2" s="15">
         <v>50</v>
       </c>
-      <c r="BF2" s="1">
+      <c r="BF2" s="57">
         <v>10</v>
       </c>
-      <c r="BG2" s="22"/>
-      <c r="BH2"/>
-      <c r="BI2"/>
-      <c r="BK2" s="13">
+      <c r="BG2" s="98"/>
+      <c r="BI2" s="15"/>
+      <c r="BK2" s="20">
         <v>1</v>
       </c>
-      <c r="BL2" s="13">
+      <c r="BL2" s="20">
         <v>0</v>
       </c>
-      <c r="BM2" s="13">
+      <c r="BM2" s="20">
         <v>50</v>
       </c>
-      <c r="BN2" s="66">
+      <c r="BN2" s="56">
         <v>10</v>
       </c>
-      <c r="BO2" s="67"/>
+      <c r="BO2" s="20">
+        <v>0</v>
+      </c>
+      <c r="BP2" s="20">
+        <v>0</v>
+      </c>
+      <c r="BQ2" s="20">
+        <v>0</v>
+      </c>
+      <c r="BR2" s="20">
+        <v>0</v>
+      </c>
+      <c r="BS2" s="20">
+        <v>0</v>
+      </c>
+      <c r="BT2" s="20">
+        <v>0</v>
+      </c>
+      <c r="BU2" s="20">
+        <v>0</v>
+      </c>
+      <c r="BV2" s="99">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:74" s="15" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="8"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="H3" s="21"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
+      <c r="N3" s="20"/>
+      <c r="O3" s="20"/>
+      <c r="P3" s="20"/>
+      <c r="Q3" s="20"/>
       <c r="R3" s="20"/>
-      <c r="AM3"/>
-      <c r="AN3"/>
-      <c r="AO3"/>
-      <c r="AP3" s="1"/>
-      <c r="BC3"/>
-      <c r="BD3"/>
-      <c r="BE3"/>
-      <c r="BF3" s="1"/>
+      <c r="S3" s="20"/>
+      <c r="T3" s="20"/>
+      <c r="U3" s="20"/>
+      <c r="V3" s="20"/>
+      <c r="W3" s="20"/>
+      <c r="X3" s="20"/>
+      <c r="Y3" s="20"/>
+      <c r="Z3" s="20"/>
+      <c r="AA3" s="20"/>
+      <c r="AB3" s="20"/>
+      <c r="AC3" s="20"/>
+      <c r="AD3" s="20"/>
+      <c r="AE3" s="20"/>
+      <c r="AF3" s="20"/>
+      <c r="AG3" s="20"/>
+      <c r="AH3" s="56"/>
+      <c r="AI3" s="98"/>
+      <c r="AL3" s="20"/>
+      <c r="AP3" s="57"/>
+      <c r="AQ3" s="98"/>
+      <c r="AT3" s="20"/>
+      <c r="AU3" s="20"/>
+      <c r="AV3" s="20"/>
+      <c r="AW3" s="20"/>
+      <c r="AX3" s="56"/>
+      <c r="AY3" s="98"/>
+      <c r="AZ3" s="20"/>
+      <c r="BA3" s="20"/>
+      <c r="BB3" s="20"/>
+      <c r="BF3" s="57"/>
+      <c r="BG3" s="98"/>
+      <c r="BH3" s="20"/>
+      <c r="BJ3" s="20"/>
+      <c r="BK3" s="20"/>
+      <c r="BL3" s="20"/>
+      <c r="BM3" s="20"/>
+      <c r="BN3" s="56"/>
+      <c r="BO3" s="20"/>
+      <c r="BP3" s="20"/>
+      <c r="BQ3" s="20"/>
+      <c r="BR3" s="20"/>
+      <c r="BS3" s="20"/>
+      <c r="BT3" s="20"/>
+      <c r="BU3" s="20"/>
+      <c r="BV3" s="100"/>
     </row>
-    <row r="4" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:74" x14ac:dyDescent="0.3">
       <c r="H4" s="21"/>
       <c r="R4" s="20"/>
+      <c r="AJ4" s="101"/>
       <c r="AM4"/>
       <c r="AN4"/>
       <c r="AO4"/>
@@ -2689,7 +2876,7 @@
       <c r="BE4"/>
       <c r="BF4" s="1"/>
     </row>
-    <row r="5" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:74" x14ac:dyDescent="0.3">
       <c r="H5" s="21"/>
       <c r="R5" s="20"/>
       <c r="AM5"/>
@@ -2701,7 +2888,7 @@
       <c r="BE5"/>
       <c r="BF5" s="1"/>
     </row>
-    <row r="6" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:74" x14ac:dyDescent="0.3">
       <c r="H6" s="21"/>
       <c r="R6" s="20"/>
       <c r="AM6"/>
@@ -2713,7 +2900,7 @@
       <c r="BE6"/>
       <c r="BF6" s="1"/>
     </row>
-    <row r="7" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:74" x14ac:dyDescent="0.3">
       <c r="H7" s="21"/>
       <c r="R7" s="20"/>
       <c r="AM7"/>
@@ -2725,7 +2912,7 @@
       <c r="BE7"/>
       <c r="BF7" s="1"/>
     </row>
-    <row r="8" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:74" x14ac:dyDescent="0.3">
       <c r="H8" s="21"/>
       <c r="R8" s="20"/>
       <c r="AM8"/>
@@ -2737,7 +2924,7 @@
       <c r="BE8"/>
       <c r="BF8" s="1"/>
     </row>
-    <row r="9" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:74" x14ac:dyDescent="0.3">
       <c r="H9" s="21"/>
       <c r="R9" s="20"/>
       <c r="AM9"/>
@@ -2749,7 +2936,7 @@
       <c r="BE9"/>
       <c r="BF9" s="1"/>
     </row>
-    <row r="10" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:74" x14ac:dyDescent="0.3">
       <c r="H10" s="21"/>
       <c r="R10" s="20"/>
       <c r="AM10"/>
@@ -2761,7 +2948,7 @@
       <c r="BE10"/>
       <c r="BF10" s="1"/>
     </row>
-    <row r="11" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:74" x14ac:dyDescent="0.3">
       <c r="H11" s="21"/>
       <c r="R11" s="20"/>
       <c r="AM11"/>
@@ -2773,7 +2960,7 @@
       <c r="BE11"/>
       <c r="BF11" s="1"/>
     </row>
-    <row r="12" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:74" x14ac:dyDescent="0.3">
       <c r="H12" s="21"/>
       <c r="R12" s="20"/>
       <c r="AM12"/>
@@ -2785,7 +2972,7 @@
       <c r="BE12"/>
       <c r="BF12" s="1"/>
     </row>
-    <row r="13" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:74" x14ac:dyDescent="0.3">
       <c r="H13" s="21"/>
       <c r="R13" s="20"/>
       <c r="AM13"/>
@@ -2797,7 +2984,7 @@
       <c r="BE13"/>
       <c r="BF13" s="1"/>
     </row>
-    <row r="14" spans="1:67" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:74" x14ac:dyDescent="0.3">
       <c r="H14" s="21"/>
       <c r="R14" s="20"/>
       <c r="AM14"/>
@@ -2818,416 +3005,440 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:BZ13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="53.1796875" style="8" customWidth="1"/>
+    <col min="1" max="1" width="53.21875" style="8" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="6.90625" customWidth="1"/>
-    <col min="5" max="5" width="8.90625" customWidth="1"/>
-    <col min="6" max="6" width="9.08984375" customWidth="1"/>
-    <col min="7" max="7" width="10.54296875" customWidth="1"/>
+    <col min="4" max="4" width="6.88671875" customWidth="1"/>
+    <col min="5" max="5" width="8.88671875" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" customWidth="1"/>
     <col min="8" max="8" width="9" style="1" customWidth="1"/>
-    <col min="9" max="9" width="8.6328125" customWidth="1"/>
-    <col min="10" max="10" width="9.453125" customWidth="1"/>
-    <col min="11" max="11" width="10.08984375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="8.6640625" customWidth="1"/>
+    <col min="10" max="10" width="9.44140625" customWidth="1"/>
+    <col min="11" max="11" width="10.109375" style="1" customWidth="1"/>
     <col min="12" max="12" width="5" customWidth="1"/>
-    <col min="13" max="13" width="8.453125" customWidth="1"/>
-    <col min="14" max="14" width="10.54296875" customWidth="1"/>
-    <col min="15" max="15" width="7.1796875" customWidth="1"/>
-    <col min="16" max="16" width="10.08984375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="4.1796875" customWidth="1"/>
+    <col min="13" max="13" width="8.44140625" customWidth="1"/>
+    <col min="14" max="14" width="10.5546875" customWidth="1"/>
+    <col min="15" max="15" width="7.21875" customWidth="1"/>
+    <col min="16" max="16" width="10.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.21875" customWidth="1"/>
     <col min="18" max="18" width="5" style="1" customWidth="1"/>
-    <col min="19" max="19" width="4.08984375" customWidth="1"/>
-    <col min="20" max="20" width="4.6328125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="4.1796875" customWidth="1"/>
+    <col min="19" max="19" width="4.109375" customWidth="1"/>
+    <col min="20" max="20" width="4.6640625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="4.21875" customWidth="1"/>
     <col min="22" max="22" width="4" style="1" customWidth="1"/>
-    <col min="23" max="23" width="4.54296875" customWidth="1"/>
+    <col min="23" max="23" width="4.5546875" customWidth="1"/>
     <col min="24" max="24" width="5" style="1" customWidth="1"/>
-    <col min="25" max="25" width="4.1796875" customWidth="1"/>
-    <col min="26" max="26" width="9.6328125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="14.6328125" style="1" customWidth="1"/>
-    <col min="28" max="28" width="15.90625" customWidth="1"/>
-    <col min="29" max="29" width="15.6328125" style="1" customWidth="1"/>
-    <col min="30" max="30" width="9.08984375" customWidth="1"/>
-    <col min="31" max="31" width="9.08984375" style="1" customWidth="1"/>
-    <col min="32" max="32" width="9.08984375" customWidth="1"/>
-    <col min="33" max="33" width="9.08984375" style="1" customWidth="1"/>
-    <col min="34" max="34" width="9.08984375" customWidth="1"/>
-    <col min="35" max="35" width="9.08984375" style="1" customWidth="1"/>
-    <col min="36" max="36" width="9.08984375" customWidth="1"/>
-    <col min="37" max="37" width="9.08984375" style="1" customWidth="1"/>
-    <col min="38" max="38" width="9.08984375" customWidth="1"/>
-    <col min="39" max="39" width="9.08984375" style="1" customWidth="1"/>
-    <col min="40" max="40" width="9.08984375" customWidth="1"/>
-    <col min="41" max="41" width="9.08984375" style="1" customWidth="1"/>
-    <col min="42" max="42" width="9.08984375" customWidth="1"/>
-    <col min="43" max="43" width="9.08984375" style="1" customWidth="1"/>
-    <col min="44" max="44" width="9.08984375" customWidth="1"/>
-    <col min="45" max="45" width="9.08984375" style="1" customWidth="1"/>
-    <col min="46" max="46" width="9.08984375" customWidth="1"/>
-    <col min="47" max="47" width="9.08984375" style="1" customWidth="1"/>
-    <col min="48" max="48" width="9.08984375" customWidth="1"/>
-    <col min="49" max="49" width="9.08984375" style="1" customWidth="1"/>
-    <col min="50" max="50" width="9.08984375" customWidth="1"/>
-    <col min="51" max="51" width="9.08984375" style="1" customWidth="1"/>
-    <col min="52" max="52" width="9.08984375" customWidth="1"/>
-    <col min="53" max="53" width="9.08984375" style="1" customWidth="1"/>
-    <col min="54" max="54" width="17.90625" customWidth="1"/>
-    <col min="55" max="55" width="9.453125" style="1" customWidth="1"/>
-    <col min="56" max="56" width="21.6328125" style="1" customWidth="1"/>
-    <col min="57" max="57" width="9.453125" style="1" customWidth="1"/>
-    <col min="58" max="58" width="21.6328125" customWidth="1"/>
-    <col min="59" max="59" width="17.90625" customWidth="1"/>
-    <col min="60" max="61" width="9.453125" style="1" customWidth="1"/>
-    <col min="62" max="62" width="21.6328125" customWidth="1"/>
-    <col min="63" max="63" width="17.90625" customWidth="1"/>
-    <col min="64" max="64" width="15.36328125" style="1" customWidth="1"/>
-    <col min="65" max="65" width="16.453125" style="1" customWidth="1"/>
-    <col min="66" max="66" width="15.1796875" style="1" customWidth="1"/>
-    <col min="67" max="67" width="18.90625" style="1" customWidth="1"/>
-    <col min="68" max="68" width="10.54296875" customWidth="1"/>
-    <col min="69" max="70" width="10.54296875" style="1" customWidth="1"/>
-    <col min="71" max="71" width="30.81640625" style="1" customWidth="1"/>
-    <col min="72" max="73" width="10.54296875" style="9" customWidth="1"/>
-    <col min="74" max="74" width="16.36328125" customWidth="1"/>
-    <col min="75" max="77" width="10.54296875" customWidth="1"/>
-    <col min="78" max="78" width="10.54296875" style="8" customWidth="1"/>
-    <col min="79" max="790" width="10.54296875" customWidth="1"/>
-    <col min="791" max="1025" width="9.08984375" customWidth="1"/>
+    <col min="25" max="25" width="4.21875" customWidth="1"/>
+    <col min="26" max="26" width="9.6640625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="14.6640625" style="1" customWidth="1"/>
+    <col min="28" max="28" width="15.88671875" customWidth="1"/>
+    <col min="29" max="29" width="15.6640625" style="1" customWidth="1"/>
+    <col min="30" max="30" width="9.109375" customWidth="1"/>
+    <col min="31" max="31" width="9.109375" style="1" customWidth="1"/>
+    <col min="32" max="32" width="9.109375" customWidth="1"/>
+    <col min="33" max="33" width="9.109375" style="1" customWidth="1"/>
+    <col min="34" max="34" width="9.109375" customWidth="1"/>
+    <col min="35" max="35" width="9.109375" style="1" customWidth="1"/>
+    <col min="36" max="36" width="9.109375" customWidth="1"/>
+    <col min="37" max="37" width="9.109375" style="1" customWidth="1"/>
+    <col min="38" max="38" width="9.109375" customWidth="1"/>
+    <col min="39" max="39" width="9.109375" style="1" customWidth="1"/>
+    <col min="40" max="40" width="9.109375" customWidth="1"/>
+    <col min="41" max="41" width="9.109375" style="1" customWidth="1"/>
+    <col min="42" max="42" width="9.109375" customWidth="1"/>
+    <col min="43" max="43" width="9.109375" style="1" customWidth="1"/>
+    <col min="44" max="44" width="9.109375" customWidth="1"/>
+    <col min="45" max="45" width="9.109375" style="1" customWidth="1"/>
+    <col min="46" max="46" width="9.109375" customWidth="1"/>
+    <col min="47" max="47" width="9.109375" style="1" customWidth="1"/>
+    <col min="48" max="48" width="9.109375" customWidth="1"/>
+    <col min="49" max="49" width="9.109375" style="1" customWidth="1"/>
+    <col min="50" max="50" width="9.109375" customWidth="1"/>
+    <col min="51" max="51" width="9.109375" style="1" customWidth="1"/>
+    <col min="52" max="52" width="9.109375" customWidth="1"/>
+    <col min="53" max="53" width="9.109375" style="1" customWidth="1"/>
+    <col min="54" max="54" width="17.88671875" customWidth="1"/>
+    <col min="55" max="55" width="9.44140625" style="1" customWidth="1"/>
+    <col min="56" max="56" width="21.6640625" style="1" customWidth="1"/>
+    <col min="57" max="57" width="9.44140625" style="1" customWidth="1"/>
+    <col min="58" max="58" width="21.6640625" customWidth="1"/>
+    <col min="59" max="59" width="17.88671875" customWidth="1"/>
+    <col min="60" max="61" width="9.44140625" style="1" customWidth="1"/>
+    <col min="62" max="62" width="21.6640625" customWidth="1"/>
+    <col min="63" max="63" width="17.88671875" customWidth="1"/>
+    <col min="64" max="64" width="15.33203125" style="1" customWidth="1"/>
+    <col min="65" max="65" width="16.44140625" style="1" customWidth="1"/>
+    <col min="66" max="66" width="15.21875" style="1" customWidth="1"/>
+    <col min="67" max="67" width="18.88671875" style="1" customWidth="1"/>
+    <col min="68" max="68" width="10.5546875" customWidth="1"/>
+    <col min="69" max="70" width="10.5546875" style="1" customWidth="1"/>
+    <col min="71" max="71" width="30.77734375" style="1" customWidth="1"/>
+    <col min="72" max="73" width="10.5546875" style="9" customWidth="1"/>
+    <col min="74" max="74" width="16.33203125" customWidth="1"/>
+    <col min="75" max="77" width="10.5546875" customWidth="1"/>
+    <col min="78" max="78" width="10.5546875" style="8" customWidth="1"/>
+    <col min="79" max="790" width="10.5546875" customWidth="1"/>
+    <col min="791" max="1025" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:78" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:78" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="47" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="G1" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="H1" s="25" t="s">
+      <c r="H1" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="I1" s="49" t="s">
+      <c r="I1" s="48" t="s">
         <v>124</v>
       </c>
-      <c r="J1" s="26" t="s">
+      <c r="J1" s="25" t="s">
         <v>125</v>
       </c>
-      <c r="K1" s="50" t="s">
+      <c r="K1" s="49" t="s">
         <v>126</v>
       </c>
-      <c r="L1" s="51" t="s">
+      <c r="L1" s="50" t="s">
         <v>127</v>
       </c>
-      <c r="M1" s="51" t="s">
+      <c r="M1" s="50" t="s">
         <v>128</v>
       </c>
-      <c r="N1" s="51" t="s">
+      <c r="N1" s="50" t="s">
         <v>129</v>
       </c>
-      <c r="O1" s="27" t="s">
+      <c r="O1" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="P1" s="38" t="s">
+      <c r="P1" s="37" t="s">
         <v>131</v>
       </c>
-      <c r="Q1" s="27" t="s">
+      <c r="Q1" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="R1" s="27" t="s">
+      <c r="R1" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="S1" s="27" t="s">
+      <c r="S1" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="T1" s="27" t="s">
+      <c r="T1" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="U1" s="27" t="s">
+      <c r="U1" s="26" t="s">
         <v>136</v>
       </c>
-      <c r="V1" s="27" t="s">
+      <c r="V1" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="W1" s="27" t="s">
+      <c r="W1" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="X1" s="27" t="s">
+      <c r="X1" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="Y1" s="27" t="s">
+      <c r="Y1" s="102" t="s">
         <v>140</v>
       </c>
-      <c r="Z1" s="38" t="s">
+      <c r="Z1" s="103" t="s">
         <v>141</v>
       </c>
-      <c r="AA1" s="23" t="s">
+      <c r="AA1" s="104" t="s">
         <v>142</v>
       </c>
-      <c r="AB1" s="23" t="s">
+      <c r="AB1" s="22" t="s">
         <v>143</v>
       </c>
-      <c r="AC1" s="28" t="s">
+      <c r="AC1" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="AD1" s="29" t="s">
+      <c r="AD1" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="AE1" s="30" t="s">
+      <c r="AE1" s="29" t="s">
         <v>146</v>
       </c>
-      <c r="AF1" s="31" t="s">
+      <c r="AF1" s="30" t="s">
         <v>147</v>
       </c>
-      <c r="AG1" s="32" t="s">
+      <c r="AG1" s="31" t="s">
         <v>148</v>
       </c>
-      <c r="AH1" s="29" t="s">
+      <c r="AH1" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="AI1" s="30" t="s">
+      <c r="AI1" s="29" t="s">
         <v>150</v>
       </c>
-      <c r="AJ1" s="31" t="s">
+      <c r="AJ1" s="30" t="s">
         <v>151</v>
       </c>
-      <c r="AK1" s="32" t="s">
+      <c r="AK1" s="31" t="s">
         <v>152</v>
       </c>
-      <c r="AL1" s="29" t="s">
+      <c r="AL1" s="28" t="s">
         <v>153</v>
       </c>
-      <c r="AM1" s="30" t="s">
+      <c r="AM1" s="29" t="s">
         <v>154</v>
       </c>
-      <c r="AN1" s="31" t="s">
+      <c r="AN1" s="30" t="s">
         <v>155</v>
       </c>
-      <c r="AO1" s="32" t="s">
+      <c r="AO1" s="31" t="s">
         <v>156</v>
       </c>
-      <c r="AP1" s="29" t="s">
+      <c r="AP1" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="AQ1" s="30" t="s">
+      <c r="AQ1" s="29" t="s">
         <v>158</v>
       </c>
-      <c r="AR1" s="31" t="s">
+      <c r="AR1" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="AS1" s="32" t="s">
+      <c r="AS1" s="31" t="s">
         <v>160</v>
       </c>
-      <c r="AT1" s="29" t="s">
+      <c r="AT1" s="28" t="s">
         <v>161</v>
       </c>
-      <c r="AU1" s="30" t="s">
+      <c r="AU1" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="AV1" s="31" t="s">
+      <c r="AV1" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="AW1" s="32" t="s">
+      <c r="AW1" s="31" t="s">
         <v>164</v>
       </c>
-      <c r="AX1" s="29" t="s">
+      <c r="AX1" s="28" t="s">
         <v>165</v>
       </c>
-      <c r="AY1" s="30" t="s">
+      <c r="AY1" s="29" t="s">
         <v>166</v>
       </c>
-      <c r="AZ1" s="31" t="s">
+      <c r="AZ1" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="BA1" s="32" t="s">
+      <c r="BA1" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="BB1" s="23" t="s">
+      <c r="BB1" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="BC1" s="23" t="s">
+      <c r="BC1" s="22" t="s">
         <v>170</v>
       </c>
-      <c r="BD1" s="52" t="s">
+      <c r="BD1" s="51" t="s">
         <v>171</v>
       </c>
-      <c r="BE1" s="33" t="s">
+      <c r="BE1" s="32" t="s">
         <v>172</v>
       </c>
-      <c r="BF1" s="33" t="s">
+      <c r="BF1" s="32" t="s">
         <v>173</v>
       </c>
-      <c r="BG1" s="53" t="s">
+      <c r="BG1" s="52" t="s">
         <v>174</v>
       </c>
-      <c r="BH1" s="34" t="s">
+      <c r="BH1" s="33" t="s">
         <v>175</v>
       </c>
-      <c r="BI1" s="47" t="s">
+      <c r="BI1" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="BJ1" s="44" t="s">
+      <c r="BJ1" s="43" t="s">
         <v>177</v>
       </c>
-      <c r="BK1" s="44" t="s">
+      <c r="BK1" s="43" t="s">
         <v>178</v>
       </c>
-      <c r="BL1" s="43" t="s">
+      <c r="BL1" s="42" t="s">
         <v>179</v>
       </c>
-      <c r="BM1" s="33" t="s">
+      <c r="BM1" s="32" t="s">
         <v>180</v>
       </c>
-      <c r="BN1" s="34" t="s">
+      <c r="BN1" s="33" t="s">
         <v>181</v>
       </c>
-      <c r="BO1" s="36" t="s">
+      <c r="BO1" s="35" t="s">
         <v>182</v>
       </c>
-      <c r="BP1" s="36" t="s">
+      <c r="BP1" s="35" t="s">
         <v>183</v>
       </c>
-      <c r="BQ1" s="37" t="s">
+      <c r="BQ1" s="36" t="s">
         <v>184</v>
       </c>
-      <c r="BR1" s="71" t="s">
+      <c r="BR1" s="66" t="s">
         <v>185</v>
       </c>
-      <c r="BS1" s="68" t="s">
+      <c r="BS1" s="63" t="s">
         <v>186</v>
       </c>
-      <c r="BT1" s="72" t="s">
+      <c r="BT1" s="67" t="s">
         <v>187</v>
       </c>
-      <c r="BU1" s="69" t="s">
+      <c r="BU1" s="64" t="s">
         <v>188</v>
       </c>
-      <c r="BV1" s="27" t="s">
+      <c r="BV1" s="26" t="s">
         <v>189</v>
       </c>
-      <c r="BW1" s="27" t="s">
+      <c r="BW1" s="26" t="s">
         <v>190</v>
       </c>
-      <c r="BX1" s="27" t="s">
+      <c r="BX1" s="26" t="s">
         <v>191</v>
       </c>
-      <c r="BY1" s="27" t="s">
+      <c r="BY1" s="26" t="s">
         <v>192</v>
       </c>
-      <c r="BZ1" s="38" t="s">
+      <c r="BZ1" s="37" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="2" spans="1:78" x14ac:dyDescent="0.35">
-      <c r="A2" s="56"/>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45">
+    <row r="2" spans="1:78" x14ac:dyDescent="0.3">
+      <c r="A2" s="105"/>
+      <c r="B2" t="s">
+        <v>246</v>
+      </c>
+      <c r="C2" t="s">
+        <v>246</v>
+      </c>
+      <c r="D2" t="s">
+        <v>246</v>
+      </c>
+      <c r="E2" t="s">
+        <v>246</v>
+      </c>
+      <c r="F2" t="s">
+        <v>246</v>
+      </c>
+      <c r="G2" t="s">
+        <v>246</v>
+      </c>
+      <c r="H2" s="107" t="s">
+        <v>246</v>
+      </c>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44">
         <v>0</v>
       </c>
-      <c r="K2" s="54"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45">
+      <c r="K2" s="53"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44">
         <v>1</v>
       </c>
-      <c r="P2" s="70">
+      <c r="P2" s="65">
         <v>2</v>
       </c>
-      <c r="Q2" s="45"/>
-      <c r="R2" s="54"/>
-      <c r="S2" s="45"/>
-      <c r="T2" s="54"/>
-      <c r="U2" s="45"/>
-      <c r="V2" s="54"/>
-      <c r="W2" s="45"/>
-      <c r="X2" s="54"/>
-      <c r="Y2" s="45"/>
-      <c r="Z2" s="54"/>
-      <c r="AA2" s="55">
+      <c r="Q2" s="44">
+        <v>999</v>
+      </c>
+      <c r="R2" s="53">
+        <v>999</v>
+      </c>
+      <c r="S2" s="44">
+        <v>999</v>
+      </c>
+      <c r="T2" s="53">
+        <v>999</v>
+      </c>
+      <c r="U2" s="44">
+        <v>999</v>
+      </c>
+      <c r="V2" s="53">
+        <v>999</v>
+      </c>
+      <c r="W2" s="44">
+        <v>999</v>
+      </c>
+      <c r="X2" s="53">
+        <v>999</v>
+      </c>
+      <c r="Y2" s="44"/>
+      <c r="Z2" s="53"/>
+      <c r="AA2" s="54">
         <v>1</v>
       </c>
-      <c r="AB2" s="55">
+      <c r="AB2" s="44">
         <v>2</v>
       </c>
-      <c r="AC2" s="54">
+      <c r="AC2" s="53">
         <v>2</v>
       </c>
-      <c r="AD2" s="45"/>
-      <c r="AE2" s="54"/>
-      <c r="AF2" s="45"/>
-      <c r="AG2" s="54"/>
-      <c r="AH2" s="45"/>
-      <c r="AI2" s="54"/>
-      <c r="AJ2" s="45"/>
-      <c r="AK2" s="54"/>
-      <c r="AL2" s="45"/>
-      <c r="AM2" s="54"/>
-      <c r="AN2" s="45"/>
-      <c r="AO2" s="54"/>
-      <c r="AP2" s="45"/>
-      <c r="AQ2" s="54"/>
-      <c r="AR2" s="45"/>
-      <c r="AS2" s="54"/>
-      <c r="AT2" s="45"/>
-      <c r="AU2" s="54"/>
-      <c r="AV2" s="45"/>
-      <c r="AW2" s="54"/>
-      <c r="AX2" s="45"/>
-      <c r="AY2" s="54"/>
-      <c r="AZ2" s="45"/>
-      <c r="BA2" s="54"/>
-      <c r="BB2" s="45">
+      <c r="AD2" s="44"/>
+      <c r="AE2" s="53"/>
+      <c r="AF2" s="44"/>
+      <c r="AG2" s="53"/>
+      <c r="AH2" s="44"/>
+      <c r="AI2" s="53"/>
+      <c r="AJ2" s="44"/>
+      <c r="AK2" s="53"/>
+      <c r="AL2" s="44"/>
+      <c r="AM2" s="53"/>
+      <c r="AN2" s="44"/>
+      <c r="AO2" s="53"/>
+      <c r="AP2" s="44"/>
+      <c r="AQ2" s="53"/>
+      <c r="AR2" s="44"/>
+      <c r="AS2" s="53"/>
+      <c r="AT2" s="44"/>
+      <c r="AU2" s="53"/>
+      <c r="AV2" s="44"/>
+      <c r="AW2" s="53"/>
+      <c r="AX2" s="44"/>
+      <c r="AY2" s="53"/>
+      <c r="AZ2" s="44"/>
+      <c r="BA2" s="53"/>
+      <c r="BB2" s="44">
         <v>1</v>
       </c>
-      <c r="BC2" s="54">
+      <c r="BC2" s="53">
         <v>0</v>
       </c>
-      <c r="BD2" s="55">
+      <c r="BD2" s="53"/>
+      <c r="BE2" s="53">
+        <v>0.11</v>
+      </c>
+      <c r="BF2" s="44">
+        <v>2</v>
+      </c>
+      <c r="BG2" s="44"/>
+      <c r="BH2" s="53">
         <v>100</v>
       </c>
-      <c r="BE2" s="54">
-        <v>0.11</v>
-      </c>
-      <c r="BF2" s="45">
-        <v>2</v>
-      </c>
-      <c r="BG2" s="45">
-        <v>1</v>
-      </c>
-      <c r="BH2" s="54">
-        <v>100</v>
-      </c>
-      <c r="BI2" s="55"/>
-      <c r="BJ2" s="45"/>
-      <c r="BK2" s="45"/>
-      <c r="BL2" s="54">
-        <v>1</v>
-      </c>
-      <c r="BM2" s="55">
-        <v>0</v>
+      <c r="BI2" s="54"/>
+      <c r="BJ2" s="44"/>
+      <c r="BK2" s="44"/>
+      <c r="BL2" s="53"/>
+      <c r="BM2" s="54">
+        <v>15</v>
       </c>
       <c r="BN2" s="54" t="s">
         <v>194</v>
@@ -3235,87 +3446,189 @@
       <c r="BO2" s="54">
         <v>1</v>
       </c>
-      <c r="BP2" s="45">
+      <c r="BP2" s="44">
         <v>1</v>
       </c>
-      <c r="BQ2" s="54">
+      <c r="BQ2" s="53">
         <v>7</v>
       </c>
-      <c r="BR2" s="70">
+      <c r="BR2" s="54">
         <v>1</v>
       </c>
       <c r="BS2" s="54">
         <v>15</v>
       </c>
-      <c r="BT2" s="55">
+      <c r="BT2" s="54">
         <v>2</v>
       </c>
-      <c r="BU2" s="55">
+      <c r="BU2" s="54">
         <v>1</v>
       </c>
-      <c r="BV2" s="45">
+      <c r="BV2" s="44">
         <v>1</v>
       </c>
-      <c r="BW2" s="45">
+      <c r="BW2" s="44">
         <v>0</v>
       </c>
-      <c r="BX2" s="45">
+      <c r="BX2" s="44">
         <v>0</v>
       </c>
-      <c r="BY2" s="45"/>
-      <c r="BZ2" s="56">
+      <c r="BY2" s="44">
         <v>0</v>
       </c>
+      <c r="BZ2" s="55">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:78" x14ac:dyDescent="0.35">
-      <c r="BD3" s="9"/>
-      <c r="BI3" s="9"/>
+    <row r="3" spans="1:78" x14ac:dyDescent="0.3">
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
+      <c r="K3" s="65"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="44"/>
+      <c r="O3" s="44"/>
+      <c r="P3" s="65"/>
+      <c r="Q3" s="44"/>
+      <c r="R3" s="65"/>
+      <c r="S3" s="44"/>
+      <c r="T3" s="65"/>
+      <c r="U3" s="44"/>
+      <c r="V3" s="65"/>
+      <c r="W3" s="44"/>
+      <c r="X3" s="65"/>
+      <c r="Y3" s="44"/>
+      <c r="Z3" s="65"/>
+      <c r="AA3" s="108"/>
+      <c r="AB3" s="44"/>
+      <c r="AC3" s="65"/>
+      <c r="AD3" s="44"/>
+      <c r="AF3" s="44"/>
+      <c r="AH3" s="44"/>
+      <c r="AJ3" s="44"/>
+      <c r="AL3" s="44"/>
+      <c r="AN3" s="44"/>
+      <c r="BB3" s="44"/>
+      <c r="BC3" s="65"/>
+      <c r="BD3" s="65"/>
+      <c r="BE3" s="108"/>
+      <c r="BF3" s="44"/>
+      <c r="BG3" s="44"/>
+      <c r="BH3" s="65"/>
+      <c r="BI3" s="108"/>
+      <c r="BJ3" s="44"/>
+      <c r="BK3" s="44"/>
+      <c r="BL3" s="65"/>
+      <c r="BM3" s="108"/>
+      <c r="BN3" s="108"/>
+      <c r="BO3" s="108"/>
+      <c r="BP3" s="44"/>
+      <c r="BQ3" s="65"/>
+      <c r="BR3" s="108"/>
+      <c r="BS3" s="108"/>
+      <c r="BT3" s="108"/>
+      <c r="BU3" s="108"/>
+      <c r="BV3" s="44"/>
+      <c r="BW3" s="44"/>
+      <c r="BX3" s="44"/>
+      <c r="BY3" s="44"/>
+      <c r="BZ3" s="106"/>
     </row>
-    <row r="4" spans="1:78" x14ac:dyDescent="0.35">
-      <c r="AA4" s="9"/>
-      <c r="BD4" s="9"/>
-      <c r="BI4" s="9"/>
+    <row r="4" spans="1:78" x14ac:dyDescent="0.3">
+      <c r="I4" s="44"/>
+      <c r="J4" s="44"/>
+      <c r="K4" s="65"/>
+      <c r="L4" s="44"/>
+      <c r="M4" s="44"/>
+      <c r="N4" s="44"/>
+      <c r="O4" s="44"/>
+      <c r="P4" s="65"/>
+      <c r="Q4" s="44"/>
+      <c r="R4" s="65"/>
+      <c r="S4" s="44"/>
+      <c r="T4" s="65"/>
+      <c r="U4" s="44"/>
+      <c r="V4" s="65"/>
+      <c r="W4" s="44"/>
+      <c r="X4" s="65"/>
+      <c r="Y4" s="44"/>
+      <c r="Z4" s="65"/>
+      <c r="AA4" s="108"/>
+      <c r="AB4" s="44"/>
+      <c r="AC4" s="65"/>
+      <c r="AD4" s="44"/>
+      <c r="AF4" s="44"/>
+      <c r="AH4" s="44"/>
+      <c r="AJ4" s="44"/>
+      <c r="AL4" s="44"/>
+      <c r="AN4" s="44"/>
+      <c r="AP4" s="44"/>
+      <c r="BB4" s="44"/>
+      <c r="BC4" s="65"/>
+      <c r="BD4" s="65"/>
+      <c r="BE4" s="65"/>
+      <c r="BF4" s="44"/>
+      <c r="BG4" s="44"/>
+      <c r="BH4" s="65"/>
+      <c r="BI4" s="108"/>
+      <c r="BJ4" s="44"/>
+      <c r="BK4" s="44"/>
+      <c r="BL4" s="65"/>
+      <c r="BM4" s="108"/>
+      <c r="BN4" s="108"/>
+      <c r="BO4" s="108"/>
+      <c r="BP4" s="44"/>
+      <c r="BQ4" s="65"/>
+      <c r="BR4" s="108"/>
+      <c r="BS4" s="108"/>
+      <c r="BT4" s="108"/>
+      <c r="BU4" s="108"/>
+      <c r="BV4" s="44"/>
+      <c r="BW4" s="44"/>
+      <c r="BX4" s="44"/>
+      <c r="BY4" s="44"/>
+      <c r="BZ4" s="106"/>
     </row>
-    <row r="5" spans="1:78" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:78" x14ac:dyDescent="0.3">
       <c r="AA5" s="9"/>
       <c r="BD5" s="9"/>
       <c r="BI5" s="9"/>
     </row>
-    <row r="6" spans="1:78" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:78" x14ac:dyDescent="0.3">
       <c r="AA6" s="9"/>
       <c r="BD6" s="9"/>
       <c r="BI6" s="9"/>
     </row>
-    <row r="7" spans="1:78" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:78" x14ac:dyDescent="0.3">
       <c r="AA7" s="9"/>
       <c r="BD7" s="9"/>
       <c r="BI7" s="9"/>
     </row>
-    <row r="8" spans="1:78" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:78" x14ac:dyDescent="0.3">
       <c r="AA8" s="9"/>
       <c r="BD8" s="9"/>
       <c r="BI8" s="9"/>
     </row>
-    <row r="9" spans="1:78" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:78" x14ac:dyDescent="0.3">
       <c r="AA9" s="9"/>
       <c r="BD9" s="9"/>
       <c r="BI9" s="9"/>
     </row>
-    <row r="10" spans="1:78" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:78" x14ac:dyDescent="0.3">
       <c r="AA10" s="9"/>
       <c r="BD10" s="9"/>
       <c r="BI10" s="9"/>
     </row>
-    <row r="11" spans="1:78" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:78" x14ac:dyDescent="0.3">
       <c r="AA11" s="9"/>
       <c r="BD11" s="9"/>
       <c r="BI11" s="9"/>
     </row>
-    <row r="12" spans="1:78" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:78" x14ac:dyDescent="0.3">
       <c r="BD12" s="9"/>
       <c r="BI12" s="9"/>
     </row>
-    <row r="13" spans="1:78" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:78" x14ac:dyDescent="0.3">
       <c r="BD13" s="9"/>
       <c r="BI13" s="9"/>
     </row>
@@ -3327,301 +3640,563 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:AQ2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AR8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.54296875" style="8" customWidth="1"/>
-    <col min="2" max="2" width="3.54296875" customWidth="1"/>
-    <col min="3" max="3" width="7.1796875" customWidth="1"/>
-    <col min="4" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="5.54296875" customWidth="1"/>
-    <col min="6" max="6" width="5.6328125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.1796875" customWidth="1"/>
-    <col min="8" max="8" width="7.6328125" customWidth="1"/>
-    <col min="9" max="9" width="13.54296875" customWidth="1"/>
-    <col min="10" max="10" width="11.08984375" customWidth="1"/>
-    <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="12" width="8.6328125" customWidth="1"/>
-    <col min="13" max="13" width="6.6328125" customWidth="1"/>
-    <col min="14" max="14" width="6.54296875" customWidth="1"/>
-    <col min="15" max="15" width="11.54296875" customWidth="1"/>
-    <col min="16" max="16" width="9.453125" customWidth="1"/>
-    <col min="17" max="17" width="7.90625" customWidth="1"/>
-    <col min="18" max="18" width="8.90625" customWidth="1"/>
-    <col min="19" max="19" width="10.54296875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="3" customWidth="1"/>
-    <col min="21" max="21" width="6.90625" customWidth="1"/>
-    <col min="22" max="22" width="6.6328125" customWidth="1"/>
-    <col min="23" max="23" width="6.90625" customWidth="1"/>
-    <col min="24" max="24" width="11.6328125" customWidth="1"/>
-    <col min="25" max="25" width="12.453125" customWidth="1"/>
-    <col min="26" max="26" width="9" style="1" customWidth="1"/>
-    <col min="27" max="27" width="9.1796875" customWidth="1"/>
-    <col min="28" max="28" width="3.90625" customWidth="1"/>
-    <col min="29" max="29" width="4" customWidth="1"/>
-    <col min="30" max="30" width="5.90625" customWidth="1"/>
-    <col min="31" max="31" width="6" customWidth="1"/>
-    <col min="32" max="32" width="8.54296875" style="1" customWidth="1"/>
-    <col min="33" max="42" width="9.36328125" customWidth="1"/>
-    <col min="43" max="43" width="9.36328125" style="8" customWidth="1"/>
-    <col min="44" max="1025" width="10.54296875" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" style="8" customWidth="1"/>
+    <col min="2" max="2" width="3.5546875" customWidth="1"/>
+    <col min="3" max="4" width="7.21875" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="5.5546875" customWidth="1"/>
+    <col min="7" max="7" width="5.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="8.21875" customWidth="1"/>
+    <col min="9" max="9" width="7.6640625" customWidth="1"/>
+    <col min="10" max="10" width="13.5546875" customWidth="1"/>
+    <col min="11" max="11" width="11.109375" customWidth="1"/>
+    <col min="12" max="12" width="10" customWidth="1"/>
+    <col min="13" max="13" width="8.6640625" customWidth="1"/>
+    <col min="14" max="14" width="6.6640625" customWidth="1"/>
+    <col min="15" max="15" width="6.5546875" customWidth="1"/>
+    <col min="16" max="16" width="11.5546875" customWidth="1"/>
+    <col min="17" max="17" width="9.44140625" customWidth="1"/>
+    <col min="18" max="18" width="7.88671875" customWidth="1"/>
+    <col min="19" max="19" width="8.88671875" customWidth="1"/>
+    <col min="20" max="20" width="10.5546875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="3" customWidth="1"/>
+    <col min="22" max="22" width="6.88671875" customWidth="1"/>
+    <col min="23" max="23" width="6.6640625" customWidth="1"/>
+    <col min="24" max="24" width="6.88671875" customWidth="1"/>
+    <col min="25" max="25" width="11.6640625" customWidth="1"/>
+    <col min="26" max="26" width="12.44140625" customWidth="1"/>
+    <col min="27" max="27" width="9" style="1" customWidth="1"/>
+    <col min="28" max="28" width="9.21875" customWidth="1"/>
+    <col min="29" max="29" width="3.88671875" customWidth="1"/>
+    <col min="30" max="30" width="4" customWidth="1"/>
+    <col min="31" max="31" width="5.88671875" customWidth="1"/>
+    <col min="32" max="32" width="6" customWidth="1"/>
+    <col min="33" max="33" width="8.5546875" style="1" customWidth="1"/>
+    <col min="34" max="43" width="9.33203125" customWidth="1"/>
+    <col min="44" max="44" width="9.33203125" style="8" customWidth="1"/>
+    <col min="45" max="1026" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="43" t="s">
+    <row r="1" spans="1:44" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="42" t="s">
         <v>195</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="34" t="s">
         <v>196</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="34" t="s">
         <v>197</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="34" t="s">
+        <v>247</v>
+      </c>
+      <c r="E1" s="43" t="s">
         <v>198</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="F1" s="34" t="s">
         <v>199</v>
       </c>
-      <c r="F1" s="47" t="s">
+      <c r="G1" s="46" t="s">
         <v>200</v>
       </c>
-      <c r="G1" s="46" t="s">
+      <c r="H1" s="45" t="s">
         <v>201</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="I1" s="22" t="s">
         <v>202</v>
       </c>
-      <c r="I1" s="23" t="s">
+      <c r="J1" s="22" t="s">
         <v>203</v>
       </c>
-      <c r="J1" s="23" t="s">
+      <c r="K1" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="K1" s="23" t="s">
+      <c r="L1" s="22" t="s">
         <v>205</v>
       </c>
-      <c r="L1" s="23" t="s">
+      <c r="M1" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="M1" s="23" t="s">
+      <c r="N1" s="22" t="s">
         <v>207</v>
       </c>
-      <c r="N1" s="23" t="s">
+      <c r="O1" s="22" t="s">
         <v>208</v>
       </c>
-      <c r="O1" s="23" t="s">
+      <c r="P1" s="22" t="s">
         <v>209</v>
       </c>
-      <c r="P1" s="23" t="s">
+      <c r="Q1" s="22" t="s">
         <v>210</v>
       </c>
-      <c r="Q1" s="23" t="s">
+      <c r="R1" s="22" t="s">
         <v>211</v>
       </c>
-      <c r="R1" s="23" t="s">
+      <c r="S1" s="22" t="s">
         <v>212</v>
       </c>
-      <c r="S1" s="28" t="s">
+      <c r="T1" s="27" t="s">
         <v>213</v>
       </c>
-      <c r="T1" s="39" t="s">
+      <c r="U1" s="38" t="s">
         <v>214</v>
       </c>
-      <c r="U1" s="39" t="s">
+      <c r="V1" s="38" t="s">
         <v>215</v>
       </c>
-      <c r="V1" s="39" t="s">
+      <c r="W1" s="38" t="s">
         <v>216</v>
       </c>
-      <c r="W1" s="39" t="s">
+      <c r="X1" s="38" t="s">
         <v>217</v>
       </c>
-      <c r="X1" s="39" t="s">
+      <c r="Y1" s="38" t="s">
         <v>218</v>
       </c>
-      <c r="Y1" s="39" t="s">
+      <c r="Z1" s="38" t="s">
         <v>219</v>
       </c>
-      <c r="Z1" s="40" t="s">
+      <c r="AA1" s="39" t="s">
         <v>220</v>
       </c>
-      <c r="AA1" s="24" t="s">
+      <c r="AB1" s="23" t="s">
         <v>221</v>
       </c>
-      <c r="AB1" s="24" t="s">
+      <c r="AC1" s="23" t="s">
         <v>222</v>
       </c>
-      <c r="AC1" s="24" t="s">
+      <c r="AD1" s="23" t="s">
         <v>223</v>
       </c>
-      <c r="AD1" s="24" t="s">
+      <c r="AE1" s="23" t="s">
         <v>224</v>
       </c>
-      <c r="AE1" s="24" t="s">
+      <c r="AF1" s="23" t="s">
         <v>225</v>
       </c>
-      <c r="AF1" s="25" t="s">
+      <c r="AG1" s="24" t="s">
         <v>226</v>
       </c>
-      <c r="AG1" s="41" t="s">
+      <c r="AH1" s="40" t="s">
         <v>227</v>
       </c>
-      <c r="AH1" s="41" t="s">
+      <c r="AI1" s="40" t="s">
         <v>228</v>
       </c>
-      <c r="AI1" s="41" t="s">
+      <c r="AJ1" s="40" t="s">
         <v>229</v>
       </c>
-      <c r="AJ1" s="41" t="s">
+      <c r="AK1" s="40" t="s">
         <v>230</v>
       </c>
-      <c r="AK1" s="41" t="s">
+      <c r="AL1" s="40" t="s">
         <v>231</v>
       </c>
-      <c r="AL1" s="41" t="s">
+      <c r="AM1" s="40" t="s">
         <v>232</v>
       </c>
-      <c r="AM1" s="41" t="s">
+      <c r="AN1" s="40" t="s">
         <v>233</v>
       </c>
-      <c r="AN1" s="41" t="s">
+      <c r="AO1" s="40" t="s">
         <v>234</v>
       </c>
-      <c r="AO1" s="41" t="s">
+      <c r="AP1" s="40" t="s">
         <v>235</v>
       </c>
-      <c r="AP1" s="41" t="s">
+      <c r="AQ1" s="40" t="s">
         <v>236</v>
       </c>
-      <c r="AQ1" s="42" t="s">
+      <c r="AR1" s="41" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.35">
-      <c r="A2" s="56"/>
-      <c r="B2" s="45">
+    <row r="2" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A2" s="105"/>
+      <c r="B2" s="44">
         <v>2.5</v>
       </c>
-      <c r="C2" s="45">
+      <c r="C2" s="44">
         <v>0</v>
       </c>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45">
+      <c r="D2" s="44">
+        <v>0</v>
+      </c>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44">
         <v>1000</v>
       </c>
-      <c r="F2" s="54"/>
-      <c r="G2" s="45">
-        <v>3</v>
-      </c>
-      <c r="H2" s="45">
+      <c r="G2" s="53"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44">
         <v>1.26</v>
       </c>
-      <c r="I2" s="45">
+      <c r="J2" s="44">
         <v>1</v>
       </c>
-      <c r="J2" s="45">
+      <c r="K2" s="44">
         <v>1</v>
       </c>
-      <c r="K2" s="45">
+      <c r="L2" s="44">
         <v>440</v>
       </c>
-      <c r="L2" s="45">
+      <c r="M2" s="44">
         <v>800</v>
       </c>
-      <c r="M2" s="45">
+      <c r="N2" s="44">
         <v>-0.5</v>
       </c>
-      <c r="N2" s="45">
+      <c r="O2" s="44">
         <v>-0.55000000000000004</v>
       </c>
-      <c r="O2" s="45">
+      <c r="P2" s="44">
         <v>500</v>
       </c>
-      <c r="P2" s="45">
+      <c r="Q2" s="44">
         <v>1.3</v>
       </c>
-      <c r="Q2" s="45">
+      <c r="R2" s="44">
         <v>0.8</v>
       </c>
-      <c r="R2" s="45">
+      <c r="S2" s="44">
         <v>1</v>
       </c>
-      <c r="S2" s="54">
+      <c r="T2" s="53">
         <v>-1.4</v>
       </c>
-      <c r="T2" s="45">
+      <c r="U2" s="44">
         <v>50</v>
       </c>
-      <c r="U2" s="45">
+      <c r="V2" s="44">
         <v>0.23</v>
       </c>
-      <c r="V2" s="45">
+      <c r="W2" s="44">
         <v>0.18</v>
       </c>
-      <c r="W2" s="45">
+      <c r="X2" s="44">
         <v>0.62</v>
       </c>
-      <c r="X2" s="45">
+      <c r="Y2" s="44">
         <v>1</v>
       </c>
-      <c r="Y2" s="45">
+      <c r="Z2" s="44">
         <v>1</v>
       </c>
-      <c r="Z2" s="54">
+      <c r="AA2" s="53">
         <v>2</v>
       </c>
-      <c r="AA2" s="45">
+      <c r="AB2" s="44">
         <v>0.7</v>
       </c>
-      <c r="AB2" s="45">
+      <c r="AC2" s="44">
         <v>6</v>
       </c>
-      <c r="AC2" s="45">
+      <c r="AD2" s="44">
         <v>0.5</v>
       </c>
-      <c r="AD2" s="45">
+      <c r="AE2" s="44">
         <v>0.16</v>
       </c>
-      <c r="AE2" s="45">
+      <c r="AF2" s="44">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="AF2" s="54">
+      <c r="AG2" s="53">
         <v>0.59</v>
       </c>
-      <c r="AG2" s="45">
+      <c r="AH2" s="44">
         <v>-2</v>
       </c>
-      <c r="AH2" s="45">
+      <c r="AI2" s="44">
         <v>1</v>
       </c>
-      <c r="AI2" s="45">
+      <c r="AJ2" s="44">
         <v>1.5</v>
       </c>
-      <c r="AJ2" s="45">
+      <c r="AK2" s="44">
         <v>2</v>
       </c>
-      <c r="AK2" s="45">
+      <c r="AL2" s="44">
         <v>0.5</v>
       </c>
-      <c r="AL2" s="45">
+      <c r="AM2" s="44">
         <v>0.01</v>
       </c>
-      <c r="AM2" s="45">
+      <c r="AN2" s="44">
         <v>100</v>
       </c>
-      <c r="AN2" s="45">
+      <c r="AO2" s="44">
         <v>0.02</v>
       </c>
-      <c r="AO2" s="45">
+      <c r="AP2" s="44">
         <v>10</v>
       </c>
-      <c r="AP2" s="45">
+      <c r="AQ2" s="44">
         <v>-0.5</v>
       </c>
-      <c r="AQ2" s="56">
+      <c r="AR2" s="55">
         <v>0</v>
       </c>
+    </row>
+    <row r="3" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="44"/>
+      <c r="O3" s="44"/>
+      <c r="P3" s="44"/>
+      <c r="Q3" s="44"/>
+      <c r="R3" s="44"/>
+      <c r="S3" s="44"/>
+      <c r="T3" s="65"/>
+      <c r="U3" s="44"/>
+      <c r="V3" s="44"/>
+      <c r="W3" s="44"/>
+      <c r="X3" s="44"/>
+      <c r="Y3" s="44"/>
+      <c r="Z3" s="44"/>
+      <c r="AA3" s="65"/>
+      <c r="AB3" s="44"/>
+      <c r="AC3" s="44"/>
+      <c r="AD3" s="44"/>
+      <c r="AE3" s="44"/>
+      <c r="AF3" s="44"/>
+      <c r="AG3" s="65"/>
+      <c r="AH3" s="44"/>
+      <c r="AI3" s="44"/>
+      <c r="AJ3" s="44"/>
+      <c r="AK3" s="44"/>
+      <c r="AL3" s="44"/>
+      <c r="AM3" s="44"/>
+      <c r="AN3" s="44"/>
+      <c r="AO3" s="44"/>
+      <c r="AP3" s="44"/>
+      <c r="AQ3" s="44"/>
+      <c r="AR3" s="106"/>
+    </row>
+    <row r="4" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="B4" s="44"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="F4" s="44"/>
+      <c r="H4" s="44"/>
+      <c r="I4" s="44"/>
+      <c r="J4" s="44"/>
+      <c r="K4" s="44"/>
+      <c r="L4" s="44"/>
+      <c r="M4" s="44"/>
+      <c r="N4" s="44"/>
+      <c r="O4" s="44"/>
+      <c r="P4" s="44"/>
+      <c r="Q4" s="44"/>
+      <c r="R4" s="44"/>
+      <c r="S4" s="44"/>
+      <c r="T4" s="65"/>
+      <c r="U4" s="44"/>
+      <c r="V4" s="44"/>
+      <c r="W4" s="44"/>
+      <c r="X4" s="44"/>
+      <c r="Y4" s="44"/>
+      <c r="Z4" s="44"/>
+      <c r="AA4" s="65"/>
+      <c r="AB4" s="44"/>
+      <c r="AC4" s="44"/>
+      <c r="AD4" s="44"/>
+      <c r="AE4" s="44"/>
+      <c r="AF4" s="44"/>
+      <c r="AG4" s="65"/>
+      <c r="AH4" s="44"/>
+      <c r="AI4" s="44"/>
+      <c r="AJ4" s="44"/>
+      <c r="AK4" s="44"/>
+      <c r="AL4" s="44"/>
+      <c r="AM4" s="44"/>
+      <c r="AN4" s="44"/>
+      <c r="AO4" s="44"/>
+      <c r="AP4" s="44"/>
+      <c r="AQ4" s="44"/>
+      <c r="AR4" s="106"/>
+    </row>
+    <row r="5" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="44"/>
+      <c r="M5" s="44"/>
+      <c r="N5" s="44"/>
+      <c r="O5" s="44"/>
+      <c r="P5" s="44"/>
+      <c r="Q5" s="44"/>
+      <c r="R5" s="44"/>
+      <c r="S5" s="44"/>
+      <c r="T5" s="65"/>
+      <c r="U5" s="44"/>
+      <c r="V5" s="44"/>
+      <c r="W5" s="44"/>
+      <c r="X5" s="44"/>
+      <c r="Y5" s="44"/>
+      <c r="Z5" s="44"/>
+      <c r="AA5" s="65"/>
+      <c r="AB5" s="44"/>
+      <c r="AC5" s="44"/>
+      <c r="AD5" s="44"/>
+      <c r="AE5" s="44"/>
+      <c r="AF5" s="44"/>
+      <c r="AG5" s="65"/>
+      <c r="AH5" s="44"/>
+      <c r="AI5" s="44"/>
+      <c r="AJ5" s="44"/>
+      <c r="AK5" s="44"/>
+      <c r="AL5" s="44"/>
+      <c r="AM5" s="44"/>
+      <c r="AN5" s="44"/>
+      <c r="AO5" s="44"/>
+      <c r="AP5" s="44"/>
+      <c r="AQ5" s="44"/>
+      <c r="AR5" s="106"/>
+    </row>
+    <row r="6" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="B6" s="44"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="44"/>
+      <c r="J6" s="44"/>
+      <c r="K6" s="44"/>
+      <c r="L6" s="44"/>
+      <c r="M6" s="44"/>
+      <c r="N6" s="44"/>
+      <c r="O6" s="44"/>
+      <c r="P6" s="44"/>
+      <c r="Q6" s="44"/>
+      <c r="R6" s="44"/>
+      <c r="S6" s="44"/>
+      <c r="T6" s="65"/>
+      <c r="U6" s="44"/>
+      <c r="V6" s="44"/>
+      <c r="W6" s="44"/>
+      <c r="X6" s="44"/>
+      <c r="Y6" s="44"/>
+      <c r="Z6" s="44"/>
+      <c r="AA6" s="65"/>
+      <c r="AB6" s="44"/>
+      <c r="AC6" s="44"/>
+      <c r="AD6" s="44"/>
+      <c r="AE6" s="44"/>
+      <c r="AF6" s="44"/>
+      <c r="AG6" s="65"/>
+      <c r="AH6" s="44"/>
+      <c r="AI6" s="44"/>
+      <c r="AJ6" s="44"/>
+      <c r="AK6" s="44"/>
+      <c r="AL6" s="44"/>
+      <c r="AM6" s="44"/>
+      <c r="AN6" s="44"/>
+      <c r="AO6" s="44"/>
+      <c r="AP6" s="44"/>
+      <c r="AQ6" s="44"/>
+      <c r="AR6" s="106"/>
+    </row>
+    <row r="7" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="B7" s="44"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
+      <c r="F7" s="44"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="44"/>
+      <c r="L7" s="44"/>
+      <c r="M7" s="44"/>
+      <c r="N7" s="44"/>
+      <c r="O7" s="44"/>
+      <c r="P7" s="44"/>
+      <c r="Q7" s="44"/>
+      <c r="R7" s="44"/>
+      <c r="S7" s="44"/>
+      <c r="T7" s="65"/>
+      <c r="U7" s="44"/>
+      <c r="V7" s="44"/>
+      <c r="W7" s="44"/>
+      <c r="X7" s="44"/>
+      <c r="Y7" s="44"/>
+      <c r="Z7" s="44"/>
+      <c r="AA7" s="65"/>
+      <c r="AB7" s="44"/>
+      <c r="AC7" s="44"/>
+      <c r="AD7" s="44"/>
+      <c r="AE7" s="44"/>
+      <c r="AF7" s="44"/>
+      <c r="AG7" s="65"/>
+      <c r="AH7" s="44"/>
+      <c r="AI7" s="44"/>
+      <c r="AJ7" s="44"/>
+      <c r="AK7" s="44"/>
+      <c r="AL7" s="44"/>
+      <c r="AM7" s="44"/>
+      <c r="AN7" s="44"/>
+      <c r="AO7" s="44"/>
+      <c r="AP7" s="44"/>
+      <c r="AQ7" s="44"/>
+      <c r="AR7" s="106"/>
+    </row>
+    <row r="8" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="B8" s="44"/>
+      <c r="C8" s="44"/>
+      <c r="D8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="44"/>
+      <c r="M8" s="44"/>
+      <c r="N8" s="44"/>
+      <c r="O8" s="44"/>
+      <c r="P8" s="44"/>
+      <c r="Q8" s="44"/>
+      <c r="R8" s="44"/>
+      <c r="S8" s="44"/>
+      <c r="T8" s="65"/>
+      <c r="U8" s="44"/>
+      <c r="V8" s="44"/>
+      <c r="W8" s="44"/>
+      <c r="X8" s="44"/>
+      <c r="Y8" s="44"/>
+      <c r="Z8" s="44"/>
+      <c r="AA8" s="65"/>
+      <c r="AB8" s="44"/>
+      <c r="AC8" s="44"/>
+      <c r="AD8" s="44"/>
+      <c r="AE8" s="44"/>
+      <c r="AF8" s="44"/>
+      <c r="AG8" s="65"/>
+      <c r="AH8" s="44"/>
+      <c r="AI8" s="44"/>
+      <c r="AJ8" s="44"/>
+      <c r="AK8" s="44"/>
+      <c r="AL8" s="44"/>
+      <c r="AM8" s="44"/>
+      <c r="AN8" s="44"/>
+      <c r="AO8" s="44"/>
+      <c r="AP8" s="44"/>
+      <c r="AQ8" s="44"/>
+      <c r="AR8" s="106"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
@@ -3632,7 +4207,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{545073CE-70C8-4069-9B47-FD0DF28CDCD4}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3641,7 +4216,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42D30E0E-A69C-4CAD-B057-D1D3B90899A8}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>